<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 07:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2B26DA2B-2CE7-4285-933C-5FDB334CFDB7}</x14:id>
+          <x14:id>{93F5BA05-9E2E-4B2E-9DAC-20A82328B860}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BC51DF1C-7D00-4A12-ABB4-270BF590EA29}</x14:id>
+          <x14:id>{911E1450-792C-4689-8818-D0B12B699F04}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5ACB6517-6DFE-40CD-9D5C-8A70E7FA1CB6}</x14:id>
+          <x14:id>{E5D1B94A-C2DA-4E3A-89B6-9BBE73A0D062}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7D6562E5-DF02-40FE-91A5-C4EB3441128C}</x14:id>
+          <x14:id>{B7391574-27F5-4DCE-A1DF-38A804F1C96F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2B26DA2B-2CE7-4285-933C-5FDB334CFDB7}">
+          <x14:cfRule type="dataBar" id="{93F5BA05-9E2E-4B2E-9DAC-20A82328B860}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BC51DF1C-7D00-4A12-ABB4-270BF590EA29}">
+          <x14:cfRule type="dataBar" id="{911E1450-792C-4689-8818-D0B12B699F04}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5ACB6517-6DFE-40CD-9D5C-8A70E7FA1CB6}">
+          <x14:cfRule type="dataBar" id="{E5D1B94A-C2DA-4E3A-89B6-9BBE73A0D062}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7D6562E5-DF02-40FE-91A5-C4EB3441128C}">
+          <x14:cfRule type="dataBar" id="{B7391574-27F5-4DCE-A1DF-38A804F1C96F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{64CFFE74-F178-44C8-A4E3-A70240FC987B}</x14:id>
+          <x14:id>{2CFC44F2-F271-4AF5-A2CC-D0BB790A7977}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2C086EFD-7665-49C3-812D-0E13675967B8}</x14:id>
+          <x14:id>{124E7361-DD04-4A49-9B75-91DBFC931F5C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5F873DBC-1E64-43DC-A8A5-4703860BC39D}</x14:id>
+          <x14:id>{F19D1F9E-6840-4B92-B0FF-BC7D3FB2E165}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4AE7B8A1-5CAB-43EB-8863-37163456C83D}</x14:id>
+          <x14:id>{119AEBFF-FBC8-487E-AA91-982915A2FFD9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{64CFFE74-F178-44C8-A4E3-A70240FC987B}">
+          <x14:cfRule type="dataBar" id="{2CFC44F2-F271-4AF5-A2CC-D0BB790A7977}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2C086EFD-7665-49C3-812D-0E13675967B8}">
+          <x14:cfRule type="dataBar" id="{124E7361-DD04-4A49-9B75-91DBFC931F5C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5F873DBC-1E64-43DC-A8A5-4703860BC39D}">
+          <x14:cfRule type="dataBar" id="{F19D1F9E-6840-4B92-B0FF-BC7D3FB2E165}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4AE7B8A1-5CAB-43EB-8863-37163456C83D}">
+          <x14:cfRule type="dataBar" id="{119AEBFF-FBC8-487E-AA91-982915A2FFD9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{93F5BA05-9E2E-4B2E-9DAC-20A82328B860}</x14:id>
+          <x14:id>{22867BA4-994C-4ACB-8AF7-2769E8641545}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{911E1450-792C-4689-8818-D0B12B699F04}</x14:id>
+          <x14:id>{547DB51B-F315-455C-8ACC-4C813B29E21A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E5D1B94A-C2DA-4E3A-89B6-9BBE73A0D062}</x14:id>
+          <x14:id>{E50069C4-3FDB-4B98-A342-BFDA826858B1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B7391574-27F5-4DCE-A1DF-38A804F1C96F}</x14:id>
+          <x14:id>{ED7E5BF9-9A22-4B62-85EC-AC5B0AA2D6F0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{93F5BA05-9E2E-4B2E-9DAC-20A82328B860}">
+          <x14:cfRule type="dataBar" id="{22867BA4-994C-4ACB-8AF7-2769E8641545}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{911E1450-792C-4689-8818-D0B12B699F04}">
+          <x14:cfRule type="dataBar" id="{547DB51B-F315-455C-8ACC-4C813B29E21A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E5D1B94A-C2DA-4E3A-89B6-9BBE73A0D062}">
+          <x14:cfRule type="dataBar" id="{E50069C4-3FDB-4B98-A342-BFDA826858B1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B7391574-27F5-4DCE-A1DF-38A804F1C96F}">
+          <x14:cfRule type="dataBar" id="{ED7E5BF9-9A22-4B62-85EC-AC5B0AA2D6F0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2CFC44F2-F271-4AF5-A2CC-D0BB790A7977}</x14:id>
+          <x14:id>{C9491AB3-CA88-4365-A09D-4B5F6344CDAB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{124E7361-DD04-4A49-9B75-91DBFC931F5C}</x14:id>
+          <x14:id>{FF7661D4-A8DA-4420-B5D9-69A9823F54F7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F19D1F9E-6840-4B92-B0FF-BC7D3FB2E165}</x14:id>
+          <x14:id>{8ACB11D4-001C-4097-A02A-760F502AC3B2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{119AEBFF-FBC8-487E-AA91-982915A2FFD9}</x14:id>
+          <x14:id>{B1AABF0B-922D-409C-A9B8-D53EAF9248A2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2CFC44F2-F271-4AF5-A2CC-D0BB790A7977}">
+          <x14:cfRule type="dataBar" id="{C9491AB3-CA88-4365-A09D-4B5F6344CDAB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{124E7361-DD04-4A49-9B75-91DBFC931F5C}">
+          <x14:cfRule type="dataBar" id="{FF7661D4-A8DA-4420-B5D9-69A9823F54F7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F19D1F9E-6840-4B92-B0FF-BC7D3FB2E165}">
+          <x14:cfRule type="dataBar" id="{8ACB11D4-001C-4097-A02A-760F502AC3B2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{119AEBFF-FBC8-487E-AA91-982915A2FFD9}">
+          <x14:cfRule type="dataBar" id="{B1AABF0B-922D-409C-A9B8-D53EAF9248A2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{22867BA4-994C-4ACB-8AF7-2769E8641545}</x14:id>
+          <x14:id>{37AA4829-89C3-4F17-BFBF-BFB92A1989D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{547DB51B-F315-455C-8ACC-4C813B29E21A}</x14:id>
+          <x14:id>{92C5FA4A-FC65-45AC-AC2F-84E38BD62F1C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E50069C4-3FDB-4B98-A342-BFDA826858B1}</x14:id>
+          <x14:id>{5F855F2D-B34B-4E23-8983-94C30F6A89C0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ED7E5BF9-9A22-4B62-85EC-AC5B0AA2D6F0}</x14:id>
+          <x14:id>{A99B1611-2EF5-49AB-AC71-7051501AA597}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{22867BA4-994C-4ACB-8AF7-2769E8641545}">
+          <x14:cfRule type="dataBar" id="{37AA4829-89C3-4F17-BFBF-BFB92A1989D0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{547DB51B-F315-455C-8ACC-4C813B29E21A}">
+          <x14:cfRule type="dataBar" id="{92C5FA4A-FC65-45AC-AC2F-84E38BD62F1C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E50069C4-3FDB-4B98-A342-BFDA826858B1}">
+          <x14:cfRule type="dataBar" id="{5F855F2D-B34B-4E23-8983-94C30F6A89C0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ED7E5BF9-9A22-4B62-85EC-AC5B0AA2D6F0}">
+          <x14:cfRule type="dataBar" id="{A99B1611-2EF5-49AB-AC71-7051501AA597}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C9491AB3-CA88-4365-A09D-4B5F6344CDAB}</x14:id>
+          <x14:id>{828BFDDD-73BD-4536-A2A1-8DC01ADA26FB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FF7661D4-A8DA-4420-B5D9-69A9823F54F7}</x14:id>
+          <x14:id>{B6839881-15A2-4767-82E8-E00450E24CA2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8ACB11D4-001C-4097-A02A-760F502AC3B2}</x14:id>
+          <x14:id>{DBCC634F-A6BF-4177-B698-46B209FA8832}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B1AABF0B-922D-409C-A9B8-D53EAF9248A2}</x14:id>
+          <x14:id>{26AB1466-C82A-4A70-B033-13341BC1198B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C9491AB3-CA88-4365-A09D-4B5F6344CDAB}">
+          <x14:cfRule type="dataBar" id="{828BFDDD-73BD-4536-A2A1-8DC01ADA26FB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FF7661D4-A8DA-4420-B5D9-69A9823F54F7}">
+          <x14:cfRule type="dataBar" id="{B6839881-15A2-4767-82E8-E00450E24CA2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8ACB11D4-001C-4097-A02A-760F502AC3B2}">
+          <x14:cfRule type="dataBar" id="{DBCC634F-A6BF-4177-B698-46B209FA8832}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B1AABF0B-922D-409C-A9B8-D53EAF9248A2}">
+          <x14:cfRule type="dataBar" id="{26AB1466-C82A-4A70-B033-13341BC1198B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{37AA4829-89C3-4F17-BFBF-BFB92A1989D0}</x14:id>
+          <x14:id>{6558CAA7-81A6-4A73-9C09-1839BBFB0861}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{92C5FA4A-FC65-45AC-AC2F-84E38BD62F1C}</x14:id>
+          <x14:id>{ADE7A4C2-28BF-47D0-9049-B4A2EC04F888}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5F855F2D-B34B-4E23-8983-94C30F6A89C0}</x14:id>
+          <x14:id>{05D9E4A6-451F-488E-A798-34E870169888}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A99B1611-2EF5-49AB-AC71-7051501AA597}</x14:id>
+          <x14:id>{241EFB40-2B35-4455-B6BB-3999F017A4AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{37AA4829-89C3-4F17-BFBF-BFB92A1989D0}">
+          <x14:cfRule type="dataBar" id="{6558CAA7-81A6-4A73-9C09-1839BBFB0861}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{92C5FA4A-FC65-45AC-AC2F-84E38BD62F1C}">
+          <x14:cfRule type="dataBar" id="{ADE7A4C2-28BF-47D0-9049-B4A2EC04F888}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5F855F2D-B34B-4E23-8983-94C30F6A89C0}">
+          <x14:cfRule type="dataBar" id="{05D9E4A6-451F-488E-A798-34E870169888}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A99B1611-2EF5-49AB-AC71-7051501AA597}">
+          <x14:cfRule type="dataBar" id="{241EFB40-2B35-4455-B6BB-3999F017A4AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{828BFDDD-73BD-4536-A2A1-8DC01ADA26FB}</x14:id>
+          <x14:id>{1A4AEC07-1A45-41A8-B37A-84B75E42CB52}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B6839881-15A2-4767-82E8-E00450E24CA2}</x14:id>
+          <x14:id>{5B215899-CE03-43E5-ADD3-1655CB01907F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DBCC634F-A6BF-4177-B698-46B209FA8832}</x14:id>
+          <x14:id>{2007D9D3-DCB5-4497-B23B-AB72FCFF8954}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{26AB1466-C82A-4A70-B033-13341BC1198B}</x14:id>
+          <x14:id>{F5D6A996-E33E-4B02-92F8-6B9600E76F27}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{828BFDDD-73BD-4536-A2A1-8DC01ADA26FB}">
+          <x14:cfRule type="dataBar" id="{1A4AEC07-1A45-41A8-B37A-84B75E42CB52}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B6839881-15A2-4767-82E8-E00450E24CA2}">
+          <x14:cfRule type="dataBar" id="{5B215899-CE03-43E5-ADD3-1655CB01907F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DBCC634F-A6BF-4177-B698-46B209FA8832}">
+          <x14:cfRule type="dataBar" id="{2007D9D3-DCB5-4497-B23B-AB72FCFF8954}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{26AB1466-C82A-4A70-B033-13341BC1198B}">
+          <x14:cfRule type="dataBar" id="{F5D6A996-E33E-4B02-92F8-6B9600E76F27}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6558CAA7-81A6-4A73-9C09-1839BBFB0861}</x14:id>
+          <x14:id>{D922939C-FE68-430D-956E-01E6F760B440}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ADE7A4C2-28BF-47D0-9049-B4A2EC04F888}</x14:id>
+          <x14:id>{A3A00990-FECB-40D1-894D-876147587068}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{05D9E4A6-451F-488E-A798-34E870169888}</x14:id>
+          <x14:id>{F7503BD0-F4E2-4356-B9D2-DDF366480EDF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{241EFB40-2B35-4455-B6BB-3999F017A4AB}</x14:id>
+          <x14:id>{3B5C383D-4C13-4A38-B7AC-09CA91DA1A8D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6558CAA7-81A6-4A73-9C09-1839BBFB0861}">
+          <x14:cfRule type="dataBar" id="{D922939C-FE68-430D-956E-01E6F760B440}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ADE7A4C2-28BF-47D0-9049-B4A2EC04F888}">
+          <x14:cfRule type="dataBar" id="{A3A00990-FECB-40D1-894D-876147587068}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{05D9E4A6-451F-488E-A798-34E870169888}">
+          <x14:cfRule type="dataBar" id="{F7503BD0-F4E2-4356-B9D2-DDF366480EDF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{241EFB40-2B35-4455-B6BB-3999F017A4AB}">
+          <x14:cfRule type="dataBar" id="{3B5C383D-4C13-4A38-B7AC-09CA91DA1A8D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1A4AEC07-1A45-41A8-B37A-84B75E42CB52}</x14:id>
+          <x14:id>{F51DB9F9-F2E2-4573-9C0E-334604964E30}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5B215899-CE03-43E5-ADD3-1655CB01907F}</x14:id>
+          <x14:id>{3379EF22-43E3-4469-B28F-C7FA5B8386A8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2007D9D3-DCB5-4497-B23B-AB72FCFF8954}</x14:id>
+          <x14:id>{6561A705-F7CF-4FEE-B511-93D612D9BE77}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F5D6A996-E33E-4B02-92F8-6B9600E76F27}</x14:id>
+          <x14:id>{A51A5A9C-7E67-4846-90DE-288DAAD1978D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1A4AEC07-1A45-41A8-B37A-84B75E42CB52}">
+          <x14:cfRule type="dataBar" id="{F51DB9F9-F2E2-4573-9C0E-334604964E30}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5B215899-CE03-43E5-ADD3-1655CB01907F}">
+          <x14:cfRule type="dataBar" id="{3379EF22-43E3-4469-B28F-C7FA5B8386A8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2007D9D3-DCB5-4497-B23B-AB72FCFF8954}">
+          <x14:cfRule type="dataBar" id="{6561A705-F7CF-4FEE-B511-93D612D9BE77}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F5D6A996-E33E-4B02-92F8-6B9600E76F27}">
+          <x14:cfRule type="dataBar" id="{A51A5A9C-7E67-4846-90DE-288DAAD1978D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D922939C-FE68-430D-956E-01E6F760B440}</x14:id>
+          <x14:id>{985AE5F0-57C1-40F0-9307-3DD085860E2C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A3A00990-FECB-40D1-894D-876147587068}</x14:id>
+          <x14:id>{7851C269-BDA5-47BB-95ED-2F9909833CB3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F7503BD0-F4E2-4356-B9D2-DDF366480EDF}</x14:id>
+          <x14:id>{61266E3D-8ABF-4AD7-A749-66D187D2FCAC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3B5C383D-4C13-4A38-B7AC-09CA91DA1A8D}</x14:id>
+          <x14:id>{A4CA2BB0-10A6-49A0-B4BF-2DC1804DFA4B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D922939C-FE68-430D-956E-01E6F760B440}">
+          <x14:cfRule type="dataBar" id="{985AE5F0-57C1-40F0-9307-3DD085860E2C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A3A00990-FECB-40D1-894D-876147587068}">
+          <x14:cfRule type="dataBar" id="{7851C269-BDA5-47BB-95ED-2F9909833CB3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F7503BD0-F4E2-4356-B9D2-DDF366480EDF}">
+          <x14:cfRule type="dataBar" id="{61266E3D-8ABF-4AD7-A749-66D187D2FCAC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3B5C383D-4C13-4A38-B7AC-09CA91DA1A8D}">
+          <x14:cfRule type="dataBar" id="{A4CA2BB0-10A6-49A0-B4BF-2DC1804DFA4B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F51DB9F9-F2E2-4573-9C0E-334604964E30}</x14:id>
+          <x14:id>{FD24B28F-F85A-47F1-8C8A-882580A4F03E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3379EF22-43E3-4469-B28F-C7FA5B8386A8}</x14:id>
+          <x14:id>{42318F27-7E00-47BA-AB1D-9BFFD6A79A84}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6561A705-F7CF-4FEE-B511-93D612D9BE77}</x14:id>
+          <x14:id>{B3E56687-E567-4BFA-A9D2-CF3EF9476CC1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A51A5A9C-7E67-4846-90DE-288DAAD1978D}</x14:id>
+          <x14:id>{93EEE184-FFCA-4CF5-9937-433D72761E9B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F51DB9F9-F2E2-4573-9C0E-334604964E30}">
+          <x14:cfRule type="dataBar" id="{FD24B28F-F85A-47F1-8C8A-882580A4F03E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3379EF22-43E3-4469-B28F-C7FA5B8386A8}">
+          <x14:cfRule type="dataBar" id="{42318F27-7E00-47BA-AB1D-9BFFD6A79A84}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6561A705-F7CF-4FEE-B511-93D612D9BE77}">
+          <x14:cfRule type="dataBar" id="{B3E56687-E567-4BFA-A9D2-CF3EF9476CC1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A51A5A9C-7E67-4846-90DE-288DAAD1978D}">
+          <x14:cfRule type="dataBar" id="{93EEE184-FFCA-4CF5-9937-433D72761E9B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{985AE5F0-57C1-40F0-9307-3DD085860E2C}</x14:id>
+          <x14:id>{EEA92587-E830-4BA3-897E-B1E5A52CFDC5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7851C269-BDA5-47BB-95ED-2F9909833CB3}</x14:id>
+          <x14:id>{15304331-B3EB-4B96-9EF2-230D3C38F965}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{61266E3D-8ABF-4AD7-A749-66D187D2FCAC}</x14:id>
+          <x14:id>{4368BC59-BD87-490B-AAEE-7DE9AC43CFE0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A4CA2BB0-10A6-49A0-B4BF-2DC1804DFA4B}</x14:id>
+          <x14:id>{833F341C-077A-415F-8588-A72A0F8954B5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{985AE5F0-57C1-40F0-9307-3DD085860E2C}">
+          <x14:cfRule type="dataBar" id="{EEA92587-E830-4BA3-897E-B1E5A52CFDC5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7851C269-BDA5-47BB-95ED-2F9909833CB3}">
+          <x14:cfRule type="dataBar" id="{15304331-B3EB-4B96-9EF2-230D3C38F965}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{61266E3D-8ABF-4AD7-A749-66D187D2FCAC}">
+          <x14:cfRule type="dataBar" id="{4368BC59-BD87-490B-AAEE-7DE9AC43CFE0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A4CA2BB0-10A6-49A0-B4BF-2DC1804DFA4B}">
+          <x14:cfRule type="dataBar" id="{833F341C-077A-415F-8588-A72A0F8954B5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FD24B28F-F85A-47F1-8C8A-882580A4F03E}</x14:id>
+          <x14:id>{F23066A3-0154-4502-98DD-65A039E62FF5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{42318F27-7E00-47BA-AB1D-9BFFD6A79A84}</x14:id>
+          <x14:id>{50272F40-7760-4624-8AD0-AA2785DFEA7B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B3E56687-E567-4BFA-A9D2-CF3EF9476CC1}</x14:id>
+          <x14:id>{DF1AF176-4D58-4D87-A29B-FC1C252B1250}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{93EEE184-FFCA-4CF5-9937-433D72761E9B}</x14:id>
+          <x14:id>{2D72F018-1291-4168-9F22-FBC76B02FE45}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FD24B28F-F85A-47F1-8C8A-882580A4F03E}">
+          <x14:cfRule type="dataBar" id="{F23066A3-0154-4502-98DD-65A039E62FF5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{42318F27-7E00-47BA-AB1D-9BFFD6A79A84}">
+          <x14:cfRule type="dataBar" id="{50272F40-7760-4624-8AD0-AA2785DFEA7B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B3E56687-E567-4BFA-A9D2-CF3EF9476CC1}">
+          <x14:cfRule type="dataBar" id="{DF1AF176-4D58-4D87-A29B-FC1C252B1250}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{93EEE184-FFCA-4CF5-9937-433D72761E9B}">
+          <x14:cfRule type="dataBar" id="{2D72F018-1291-4168-9F22-FBC76B02FE45}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EEA92587-E830-4BA3-897E-B1E5A52CFDC5}</x14:id>
+          <x14:id>{59073F20-67BC-437D-B228-D52D1FCBDC7D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{15304331-B3EB-4B96-9EF2-230D3C38F965}</x14:id>
+          <x14:id>{08210DFE-67B1-4579-8C59-94F8AFFF6053}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4368BC59-BD87-490B-AAEE-7DE9AC43CFE0}</x14:id>
+          <x14:id>{0B0F526F-59D9-4499-A161-6E7ECB98407D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{833F341C-077A-415F-8588-A72A0F8954B5}</x14:id>
+          <x14:id>{4C265BF4-C5C6-4BDD-86DA-D97B30E947F2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EEA92587-E830-4BA3-897E-B1E5A52CFDC5}">
+          <x14:cfRule type="dataBar" id="{59073F20-67BC-437D-B228-D52D1FCBDC7D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{15304331-B3EB-4B96-9EF2-230D3C38F965}">
+          <x14:cfRule type="dataBar" id="{08210DFE-67B1-4579-8C59-94F8AFFF6053}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4368BC59-BD87-490B-AAEE-7DE9AC43CFE0}">
+          <x14:cfRule type="dataBar" id="{0B0F526F-59D9-4499-A161-6E7ECB98407D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{833F341C-077A-415F-8588-A72A0F8954B5}">
+          <x14:cfRule type="dataBar" id="{4C265BF4-C5C6-4BDD-86DA-D97B30E947F2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F23066A3-0154-4502-98DD-65A039E62FF5}</x14:id>
+          <x14:id>{B593FE18-FD98-4F3A-863D-4AE6857F1FAC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{50272F40-7760-4624-8AD0-AA2785DFEA7B}</x14:id>
+          <x14:id>{97C2A925-1F34-453B-830A-FB48AF52D55E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DF1AF176-4D58-4D87-A29B-FC1C252B1250}</x14:id>
+          <x14:id>{A7F91F7D-F08F-4D29-A914-BAF94A600404}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2D72F018-1291-4168-9F22-FBC76B02FE45}</x14:id>
+          <x14:id>{B6C0B486-B84B-4B69-B459-5B5824E5B674}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F23066A3-0154-4502-98DD-65A039E62FF5}">
+          <x14:cfRule type="dataBar" id="{B593FE18-FD98-4F3A-863D-4AE6857F1FAC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{50272F40-7760-4624-8AD0-AA2785DFEA7B}">
+          <x14:cfRule type="dataBar" id="{97C2A925-1F34-453B-830A-FB48AF52D55E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DF1AF176-4D58-4D87-A29B-FC1C252B1250}">
+          <x14:cfRule type="dataBar" id="{A7F91F7D-F08F-4D29-A914-BAF94A600404}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2D72F018-1291-4168-9F22-FBC76B02FE45}">
+          <x14:cfRule type="dataBar" id="{B6C0B486-B84B-4B69-B459-5B5824E5B674}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{59073F20-67BC-437D-B228-D52D1FCBDC7D}</x14:id>
+          <x14:id>{C30BFC21-3F65-43E7-9A16-B7769EDD4B3A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{08210DFE-67B1-4579-8C59-94F8AFFF6053}</x14:id>
+          <x14:id>{9F0B930F-867B-4288-B652-DC45E0FD59E1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0B0F526F-59D9-4499-A161-6E7ECB98407D}</x14:id>
+          <x14:id>{5898F2FA-0AD0-4C7C-ACEF-DE647CDCC5C7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4C265BF4-C5C6-4BDD-86DA-D97B30E947F2}</x14:id>
+          <x14:id>{9FFB2D74-B3D4-4CC3-9920-8269C4ECE8AC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{59073F20-67BC-437D-B228-D52D1FCBDC7D}">
+          <x14:cfRule type="dataBar" id="{C30BFC21-3F65-43E7-9A16-B7769EDD4B3A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{08210DFE-67B1-4579-8C59-94F8AFFF6053}">
+          <x14:cfRule type="dataBar" id="{9F0B930F-867B-4288-B652-DC45E0FD59E1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0B0F526F-59D9-4499-A161-6E7ECB98407D}">
+          <x14:cfRule type="dataBar" id="{5898F2FA-0AD0-4C7C-ACEF-DE647CDCC5C7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4C265BF4-C5C6-4BDD-86DA-D97B30E947F2}">
+          <x14:cfRule type="dataBar" id="{9FFB2D74-B3D4-4CC3-9920-8269C4ECE8AC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B593FE18-FD98-4F3A-863D-4AE6857F1FAC}</x14:id>
+          <x14:id>{F89293D4-DB0B-415D-A0E6-8888722A6162}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{97C2A925-1F34-453B-830A-FB48AF52D55E}</x14:id>
+          <x14:id>{82A7F737-6BCA-41D3-BC05-E3F4AA2AFC0C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A7F91F7D-F08F-4D29-A914-BAF94A600404}</x14:id>
+          <x14:id>{4DA5B443-73E3-4E25-B25A-A4CA9781C658}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B6C0B486-B84B-4B69-B459-5B5824E5B674}</x14:id>
+          <x14:id>{FD471E01-592D-4979-AC5A-6FC43F68700C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B593FE18-FD98-4F3A-863D-4AE6857F1FAC}">
+          <x14:cfRule type="dataBar" id="{F89293D4-DB0B-415D-A0E6-8888722A6162}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{97C2A925-1F34-453B-830A-FB48AF52D55E}">
+          <x14:cfRule type="dataBar" id="{82A7F737-6BCA-41D3-BC05-E3F4AA2AFC0C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A7F91F7D-F08F-4D29-A914-BAF94A600404}">
+          <x14:cfRule type="dataBar" id="{4DA5B443-73E3-4E25-B25A-A4CA9781C658}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B6C0B486-B84B-4B69-B459-5B5824E5B674}">
+          <x14:cfRule type="dataBar" id="{FD471E01-592D-4979-AC5A-6FC43F68700C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C30BFC21-3F65-43E7-9A16-B7769EDD4B3A}</x14:id>
+          <x14:id>{F6A34AAC-E5BF-4374-B836-8A988E751F73}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9F0B930F-867B-4288-B652-DC45E0FD59E1}</x14:id>
+          <x14:id>{881A2AB4-3C81-4965-9F5C-7DCB78B56ED2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5898F2FA-0AD0-4C7C-ACEF-DE647CDCC5C7}</x14:id>
+          <x14:id>{45FF5592-E415-4130-9AF2-0182F42CEDE6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9FFB2D74-B3D4-4CC3-9920-8269C4ECE8AC}</x14:id>
+          <x14:id>{0094FB46-1DAC-4821-901D-B36D56446305}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C30BFC21-3F65-43E7-9A16-B7769EDD4B3A}">
+          <x14:cfRule type="dataBar" id="{F6A34AAC-E5BF-4374-B836-8A988E751F73}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9F0B930F-867B-4288-B652-DC45E0FD59E1}">
+          <x14:cfRule type="dataBar" id="{881A2AB4-3C81-4965-9F5C-7DCB78B56ED2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5898F2FA-0AD0-4C7C-ACEF-DE647CDCC5C7}">
+          <x14:cfRule type="dataBar" id="{45FF5592-E415-4130-9AF2-0182F42CEDE6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9FFB2D74-B3D4-4CC3-9920-8269C4ECE8AC}">
+          <x14:cfRule type="dataBar" id="{0094FB46-1DAC-4821-901D-B36D56446305}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F89293D4-DB0B-415D-A0E6-8888722A6162}</x14:id>
+          <x14:id>{87BFC1C6-CDA4-47A9-84FD-E9A62F0AC8CF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{82A7F737-6BCA-41D3-BC05-E3F4AA2AFC0C}</x14:id>
+          <x14:id>{9A6946E9-56E2-4B4E-894F-03126CC5DFF0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4DA5B443-73E3-4E25-B25A-A4CA9781C658}</x14:id>
+          <x14:id>{6A8BEE15-B2A7-4363-84D3-D57771882512}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FD471E01-592D-4979-AC5A-6FC43F68700C}</x14:id>
+          <x14:id>{CBEDFD24-AB6E-46DC-8105-7C0F58377FCB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F89293D4-DB0B-415D-A0E6-8888722A6162}">
+          <x14:cfRule type="dataBar" id="{87BFC1C6-CDA4-47A9-84FD-E9A62F0AC8CF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{82A7F737-6BCA-41D3-BC05-E3F4AA2AFC0C}">
+          <x14:cfRule type="dataBar" id="{9A6946E9-56E2-4B4E-894F-03126CC5DFF0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4DA5B443-73E3-4E25-B25A-A4CA9781C658}">
+          <x14:cfRule type="dataBar" id="{6A8BEE15-B2A7-4363-84D3-D57771882512}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FD471E01-592D-4979-AC5A-6FC43F68700C}">
+          <x14:cfRule type="dataBar" id="{CBEDFD24-AB6E-46DC-8105-7C0F58377FCB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F6A34AAC-E5BF-4374-B836-8A988E751F73}</x14:id>
+          <x14:id>{C8E1A289-4B27-4631-94CD-C79F0AF4ABDF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{881A2AB4-3C81-4965-9F5C-7DCB78B56ED2}</x14:id>
+          <x14:id>{013ED8E3-8D8B-4D1F-9D16-7C52D63D0008}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{45FF5592-E415-4130-9AF2-0182F42CEDE6}</x14:id>
+          <x14:id>{1A51D65D-4623-4D4C-B431-DF4A7C1A7401}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0094FB46-1DAC-4821-901D-B36D56446305}</x14:id>
+          <x14:id>{81A36B90-F592-4A2D-9BFE-B79DF88B2BEA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F6A34AAC-E5BF-4374-B836-8A988E751F73}">
+          <x14:cfRule type="dataBar" id="{C8E1A289-4B27-4631-94CD-C79F0AF4ABDF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{881A2AB4-3C81-4965-9F5C-7DCB78B56ED2}">
+          <x14:cfRule type="dataBar" id="{013ED8E3-8D8B-4D1F-9D16-7C52D63D0008}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{45FF5592-E415-4130-9AF2-0182F42CEDE6}">
+          <x14:cfRule type="dataBar" id="{1A51D65D-4623-4D4C-B431-DF4A7C1A7401}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0094FB46-1DAC-4821-901D-B36D56446305}">
+          <x14:cfRule type="dataBar" id="{81A36B90-F592-4A2D-9BFE-B79DF88B2BEA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{87BFC1C6-CDA4-47A9-84FD-E9A62F0AC8CF}</x14:id>
+          <x14:id>{684793AC-0C90-4683-AABA-61E7B5FFDEB1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9A6946E9-56E2-4B4E-894F-03126CC5DFF0}</x14:id>
+          <x14:id>{3195DBC7-7BA9-4FA0-B5BE-0EAE84578049}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6A8BEE15-B2A7-4363-84D3-D57771882512}</x14:id>
+          <x14:id>{27728D3E-EC02-44D5-B033-8B0E43E17FBE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CBEDFD24-AB6E-46DC-8105-7C0F58377FCB}</x14:id>
+          <x14:id>{73240A00-674B-4A89-BF92-BA82DD412ED5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{87BFC1C6-CDA4-47A9-84FD-E9A62F0AC8CF}">
+          <x14:cfRule type="dataBar" id="{684793AC-0C90-4683-AABA-61E7B5FFDEB1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9A6946E9-56E2-4B4E-894F-03126CC5DFF0}">
+          <x14:cfRule type="dataBar" id="{3195DBC7-7BA9-4FA0-B5BE-0EAE84578049}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6A8BEE15-B2A7-4363-84D3-D57771882512}">
+          <x14:cfRule type="dataBar" id="{27728D3E-EC02-44D5-B033-8B0E43E17FBE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CBEDFD24-AB6E-46DC-8105-7C0F58377FCB}">
+          <x14:cfRule type="dataBar" id="{73240A00-674B-4A89-BF92-BA82DD412ED5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C8E1A289-4B27-4631-94CD-C79F0AF4ABDF}</x14:id>
+          <x14:id>{09FFE5B2-01D8-4C5E-9B03-8413ED5CB7F1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{013ED8E3-8D8B-4D1F-9D16-7C52D63D0008}</x14:id>
+          <x14:id>{A8F3DCC6-E4C5-4B03-92A5-DA5A7A4DCEF4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1A51D65D-4623-4D4C-B431-DF4A7C1A7401}</x14:id>
+          <x14:id>{975EBC48-1090-48D8-A6D1-3699303815F6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{81A36B90-F592-4A2D-9BFE-B79DF88B2BEA}</x14:id>
+          <x14:id>{C80640CA-D985-4BF7-B710-7356A8225639}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C8E1A289-4B27-4631-94CD-C79F0AF4ABDF}">
+          <x14:cfRule type="dataBar" id="{09FFE5B2-01D8-4C5E-9B03-8413ED5CB7F1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{013ED8E3-8D8B-4D1F-9D16-7C52D63D0008}">
+          <x14:cfRule type="dataBar" id="{A8F3DCC6-E4C5-4B03-92A5-DA5A7A4DCEF4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1A51D65D-4623-4D4C-B431-DF4A7C1A7401}">
+          <x14:cfRule type="dataBar" id="{975EBC48-1090-48D8-A6D1-3699303815F6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{81A36B90-F592-4A2D-9BFE-B79DF88B2BEA}">
+          <x14:cfRule type="dataBar" id="{C80640CA-D985-4BF7-B710-7356A8225639}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{684793AC-0C90-4683-AABA-61E7B5FFDEB1}</x14:id>
+          <x14:id>{159764DD-5714-4295-A2D2-1536914A0B02}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3195DBC7-7BA9-4FA0-B5BE-0EAE84578049}</x14:id>
+          <x14:id>{76AB00A3-CF32-493F-A31E-917D96328C7A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{27728D3E-EC02-44D5-B033-8B0E43E17FBE}</x14:id>
+          <x14:id>{0F94A048-C98D-4C9F-9B9D-562A3E2604B0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{73240A00-674B-4A89-BF92-BA82DD412ED5}</x14:id>
+          <x14:id>{2D4897E8-CEB5-4CC6-9CC0-957A87762F81}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{684793AC-0C90-4683-AABA-61E7B5FFDEB1}">
+          <x14:cfRule type="dataBar" id="{159764DD-5714-4295-A2D2-1536914A0B02}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3195DBC7-7BA9-4FA0-B5BE-0EAE84578049}">
+          <x14:cfRule type="dataBar" id="{76AB00A3-CF32-493F-A31E-917D96328C7A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{27728D3E-EC02-44D5-B033-8B0E43E17FBE}">
+          <x14:cfRule type="dataBar" id="{0F94A048-C98D-4C9F-9B9D-562A3E2604B0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{73240A00-674B-4A89-BF92-BA82DD412ED5}">
+          <x14:cfRule type="dataBar" id="{2D4897E8-CEB5-4CC6-9CC0-957A87762F81}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 08:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{09FFE5B2-01D8-4C5E-9B03-8413ED5CB7F1}</x14:id>
+          <x14:id>{48869F5C-C01B-46CA-A513-D055522E04E9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A8F3DCC6-E4C5-4B03-92A5-DA5A7A4DCEF4}</x14:id>
+          <x14:id>{726C1DCB-01F8-4D54-AFD7-7FA06ABF5E54}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{975EBC48-1090-48D8-A6D1-3699303815F6}</x14:id>
+          <x14:id>{D0405756-2C15-4B37-B556-79C6B5550102}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C80640CA-D985-4BF7-B710-7356A8225639}</x14:id>
+          <x14:id>{DDC7DC81-DF6D-4D43-B554-50D11F3F3A39}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{09FFE5B2-01D8-4C5E-9B03-8413ED5CB7F1}">
+          <x14:cfRule type="dataBar" id="{48869F5C-C01B-46CA-A513-D055522E04E9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A8F3DCC6-E4C5-4B03-92A5-DA5A7A4DCEF4}">
+          <x14:cfRule type="dataBar" id="{726C1DCB-01F8-4D54-AFD7-7FA06ABF5E54}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{975EBC48-1090-48D8-A6D1-3699303815F6}">
+          <x14:cfRule type="dataBar" id="{D0405756-2C15-4B37-B556-79C6B5550102}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C80640CA-D985-4BF7-B710-7356A8225639}">
+          <x14:cfRule type="dataBar" id="{DDC7DC81-DF6D-4D43-B554-50D11F3F3A39}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{159764DD-5714-4295-A2D2-1536914A0B02}</x14:id>
+          <x14:id>{AACDC9EA-4A94-45B7-90D6-A53FC4A3BFE3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{76AB00A3-CF32-493F-A31E-917D96328C7A}</x14:id>
+          <x14:id>{4C265D0F-2DD2-4468-B454-A871BB50D9A6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0F94A048-C98D-4C9F-9B9D-562A3E2604B0}</x14:id>
+          <x14:id>{E71D7FF0-5631-4FAB-A421-49F6D10C4F21}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2D4897E8-CEB5-4CC6-9CC0-957A87762F81}</x14:id>
+          <x14:id>{185CBC0E-1912-4681-9C62-38BC8F0762D1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{159764DD-5714-4295-A2D2-1536914A0B02}">
+          <x14:cfRule type="dataBar" id="{AACDC9EA-4A94-45B7-90D6-A53FC4A3BFE3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{76AB00A3-CF32-493F-A31E-917D96328C7A}">
+          <x14:cfRule type="dataBar" id="{4C265D0F-2DD2-4468-B454-A871BB50D9A6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0F94A048-C98D-4C9F-9B9D-562A3E2604B0}">
+          <x14:cfRule type="dataBar" id="{E71D7FF0-5631-4FAB-A421-49F6D10C4F21}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2D4897E8-CEB5-4CC6-9CC0-957A87762F81}">
+          <x14:cfRule type="dataBar" id="{185CBC0E-1912-4681-9C62-38BC8F0762D1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{48869F5C-C01B-46CA-A513-D055522E04E9}</x14:id>
+          <x14:id>{FE42B6B4-DC7B-4676-9005-644CD6041922}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{726C1DCB-01F8-4D54-AFD7-7FA06ABF5E54}</x14:id>
+          <x14:id>{3917B9C9-BCD2-4385-ABD2-63909AF63C8D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D0405756-2C15-4B37-B556-79C6B5550102}</x14:id>
+          <x14:id>{DDE508E5-053B-421E-A87C-71E00064EE4D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DDC7DC81-DF6D-4D43-B554-50D11F3F3A39}</x14:id>
+          <x14:id>{5CD43E04-3A2A-4484-B933-BAE75182BC7D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{48869F5C-C01B-46CA-A513-D055522E04E9}">
+          <x14:cfRule type="dataBar" id="{FE42B6B4-DC7B-4676-9005-644CD6041922}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{726C1DCB-01F8-4D54-AFD7-7FA06ABF5E54}">
+          <x14:cfRule type="dataBar" id="{3917B9C9-BCD2-4385-ABD2-63909AF63C8D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D0405756-2C15-4B37-B556-79C6B5550102}">
+          <x14:cfRule type="dataBar" id="{DDE508E5-053B-421E-A87C-71E00064EE4D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DDC7DC81-DF6D-4D43-B554-50D11F3F3A39}">
+          <x14:cfRule type="dataBar" id="{5CD43E04-3A2A-4484-B933-BAE75182BC7D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AACDC9EA-4A94-45B7-90D6-A53FC4A3BFE3}</x14:id>
+          <x14:id>{98CE99C1-BD18-4818-9FA3-51AEA687E03A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4C265D0F-2DD2-4468-B454-A871BB50D9A6}</x14:id>
+          <x14:id>{E3E92C27-D03C-4003-A3E0-B3A33D9E449F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E71D7FF0-5631-4FAB-A421-49F6D10C4F21}</x14:id>
+          <x14:id>{56CAF786-9655-4457-A454-4C58038F2C40}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{185CBC0E-1912-4681-9C62-38BC8F0762D1}</x14:id>
+          <x14:id>{5B68CA06-C0F3-424B-BEB3-2BCE560320EC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AACDC9EA-4A94-45B7-90D6-A53FC4A3BFE3}">
+          <x14:cfRule type="dataBar" id="{98CE99C1-BD18-4818-9FA3-51AEA687E03A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4C265D0F-2DD2-4468-B454-A871BB50D9A6}">
+          <x14:cfRule type="dataBar" id="{E3E92C27-D03C-4003-A3E0-B3A33D9E449F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E71D7FF0-5631-4FAB-A421-49F6D10C4F21}">
+          <x14:cfRule type="dataBar" id="{56CAF786-9655-4457-A454-4C58038F2C40}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{185CBC0E-1912-4681-9C62-38BC8F0762D1}">
+          <x14:cfRule type="dataBar" id="{5B68CA06-C0F3-424B-BEB3-2BCE560320EC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FE42B6B4-DC7B-4676-9005-644CD6041922}</x14:id>
+          <x14:id>{F8E8A901-9794-4D34-940C-014586561BAB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3917B9C9-BCD2-4385-ABD2-63909AF63C8D}</x14:id>
+          <x14:id>{A4DEB157-4EBC-490C-B5C7-CB38CD9B21B4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DDE508E5-053B-421E-A87C-71E00064EE4D}</x14:id>
+          <x14:id>{E9033401-0D1B-4181-9A29-CD8CFDF951C9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5CD43E04-3A2A-4484-B933-BAE75182BC7D}</x14:id>
+          <x14:id>{D5823450-1609-44E0-80FC-4652E72A7A87}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FE42B6B4-DC7B-4676-9005-644CD6041922}">
+          <x14:cfRule type="dataBar" id="{F8E8A901-9794-4D34-940C-014586561BAB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3917B9C9-BCD2-4385-ABD2-63909AF63C8D}">
+          <x14:cfRule type="dataBar" id="{A4DEB157-4EBC-490C-B5C7-CB38CD9B21B4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DDE508E5-053B-421E-A87C-71E00064EE4D}">
+          <x14:cfRule type="dataBar" id="{E9033401-0D1B-4181-9A29-CD8CFDF951C9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5CD43E04-3A2A-4484-B933-BAE75182BC7D}">
+          <x14:cfRule type="dataBar" id="{D5823450-1609-44E0-80FC-4652E72A7A87}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{98CE99C1-BD18-4818-9FA3-51AEA687E03A}</x14:id>
+          <x14:id>{0D81EDC3-3935-423F-AB36-F378701ED24F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E3E92C27-D03C-4003-A3E0-B3A33D9E449F}</x14:id>
+          <x14:id>{86F9D911-6BB8-4598-AC3C-40CF4EABE831}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{56CAF786-9655-4457-A454-4C58038F2C40}</x14:id>
+          <x14:id>{FC0A5472-05B2-4BB8-BFAC-1742D7F43EE0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5B68CA06-C0F3-424B-BEB3-2BCE560320EC}</x14:id>
+          <x14:id>{81081065-0155-4F21-9D14-6ECAB551AD14}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{98CE99C1-BD18-4818-9FA3-51AEA687E03A}">
+          <x14:cfRule type="dataBar" id="{0D81EDC3-3935-423F-AB36-F378701ED24F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E3E92C27-D03C-4003-A3E0-B3A33D9E449F}">
+          <x14:cfRule type="dataBar" id="{86F9D911-6BB8-4598-AC3C-40CF4EABE831}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{56CAF786-9655-4457-A454-4C58038F2C40}">
+          <x14:cfRule type="dataBar" id="{FC0A5472-05B2-4BB8-BFAC-1742D7F43EE0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5B68CA06-C0F3-424B-BEB3-2BCE560320EC}">
+          <x14:cfRule type="dataBar" id="{81081065-0155-4F21-9D14-6ECAB551AD14}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F8E8A901-9794-4D34-940C-014586561BAB}</x14:id>
+          <x14:id>{29E425F6-657B-4BEE-87D4-D46981E4CEC7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A4DEB157-4EBC-490C-B5C7-CB38CD9B21B4}</x14:id>
+          <x14:id>{B9922996-EABA-44B1-94D3-CF80FC338A1E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E9033401-0D1B-4181-9A29-CD8CFDF951C9}</x14:id>
+          <x14:id>{22C8B3AF-C795-4071-899F-602338A7D831}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D5823450-1609-44E0-80FC-4652E72A7A87}</x14:id>
+          <x14:id>{12C1F788-F436-4FCF-BFC9-E8607DEEAE6D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F8E8A901-9794-4D34-940C-014586561BAB}">
+          <x14:cfRule type="dataBar" id="{29E425F6-657B-4BEE-87D4-D46981E4CEC7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A4DEB157-4EBC-490C-B5C7-CB38CD9B21B4}">
+          <x14:cfRule type="dataBar" id="{B9922996-EABA-44B1-94D3-CF80FC338A1E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E9033401-0D1B-4181-9A29-CD8CFDF951C9}">
+          <x14:cfRule type="dataBar" id="{22C8B3AF-C795-4071-899F-602338A7D831}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D5823450-1609-44E0-80FC-4652E72A7A87}">
+          <x14:cfRule type="dataBar" id="{12C1F788-F436-4FCF-BFC9-E8607DEEAE6D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0D81EDC3-3935-423F-AB36-F378701ED24F}</x14:id>
+          <x14:id>{1A2C379E-49FC-437C-B426-60672FF7A21A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{86F9D911-6BB8-4598-AC3C-40CF4EABE831}</x14:id>
+          <x14:id>{84095722-7F4F-4141-9407-E1C9D4304DC3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FC0A5472-05B2-4BB8-BFAC-1742D7F43EE0}</x14:id>
+          <x14:id>{5C69F042-0944-4CFD-AAC3-C10EA1900A2F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{81081065-0155-4F21-9D14-6ECAB551AD14}</x14:id>
+          <x14:id>{369B6414-AB2A-4ACD-BA1D-461EC869D092}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0D81EDC3-3935-423F-AB36-F378701ED24F}">
+          <x14:cfRule type="dataBar" id="{1A2C379E-49FC-437C-B426-60672FF7A21A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{86F9D911-6BB8-4598-AC3C-40CF4EABE831}">
+          <x14:cfRule type="dataBar" id="{84095722-7F4F-4141-9407-E1C9D4304DC3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FC0A5472-05B2-4BB8-BFAC-1742D7F43EE0}">
+          <x14:cfRule type="dataBar" id="{5C69F042-0944-4CFD-AAC3-C10EA1900A2F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{81081065-0155-4F21-9D14-6ECAB551AD14}">
+          <x14:cfRule type="dataBar" id="{369B6414-AB2A-4ACD-BA1D-461EC869D092}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{29E425F6-657B-4BEE-87D4-D46981E4CEC7}</x14:id>
+          <x14:id>{DC79E82F-C20D-4114-B449-C25DC7EF690A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B9922996-EABA-44B1-94D3-CF80FC338A1E}</x14:id>
+          <x14:id>{9E082B04-E31F-46EB-89B0-41093CD057AF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{22C8B3AF-C795-4071-899F-602338A7D831}</x14:id>
+          <x14:id>{0C5285DE-770C-4BA1-B699-FB1D33570C86}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{12C1F788-F436-4FCF-BFC9-E8607DEEAE6D}</x14:id>
+          <x14:id>{44C26EEA-516F-4C9A-86A5-53AE2A2A8895}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{29E425F6-657B-4BEE-87D4-D46981E4CEC7}">
+          <x14:cfRule type="dataBar" id="{DC79E82F-C20D-4114-B449-C25DC7EF690A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B9922996-EABA-44B1-94D3-CF80FC338A1E}">
+          <x14:cfRule type="dataBar" id="{9E082B04-E31F-46EB-89B0-41093CD057AF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{22C8B3AF-C795-4071-899F-602338A7D831}">
+          <x14:cfRule type="dataBar" id="{0C5285DE-770C-4BA1-B699-FB1D33570C86}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{12C1F788-F436-4FCF-BFC9-E8607DEEAE6D}">
+          <x14:cfRule type="dataBar" id="{44C26EEA-516F-4C9A-86A5-53AE2A2A8895}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1A2C379E-49FC-437C-B426-60672FF7A21A}</x14:id>
+          <x14:id>{6DCD2F68-D2C5-40AA-85E7-192FE793A81C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{84095722-7F4F-4141-9407-E1C9D4304DC3}</x14:id>
+          <x14:id>{A9B315FE-6419-406D-A826-4D5E1A4CBB4E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5C69F042-0944-4CFD-AAC3-C10EA1900A2F}</x14:id>
+          <x14:id>{7514BC41-566E-4EBC-BC4B-7A7CD1F0933A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{369B6414-AB2A-4ACD-BA1D-461EC869D092}</x14:id>
+          <x14:id>{DA219EC9-98F7-4F3E-AD66-A6EFC67A3121}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1A2C379E-49FC-437C-B426-60672FF7A21A}">
+          <x14:cfRule type="dataBar" id="{6DCD2F68-D2C5-40AA-85E7-192FE793A81C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{84095722-7F4F-4141-9407-E1C9D4304DC3}">
+          <x14:cfRule type="dataBar" id="{A9B315FE-6419-406D-A826-4D5E1A4CBB4E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5C69F042-0944-4CFD-AAC3-C10EA1900A2F}">
+          <x14:cfRule type="dataBar" id="{7514BC41-566E-4EBC-BC4B-7A7CD1F0933A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{369B6414-AB2A-4ACD-BA1D-461EC869D092}">
+          <x14:cfRule type="dataBar" id="{DA219EC9-98F7-4F3E-AD66-A6EFC67A3121}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DC79E82F-C20D-4114-B449-C25DC7EF690A}</x14:id>
+          <x14:id>{839CA61E-1EE3-405E-A487-E68717692F37}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9E082B04-E31F-46EB-89B0-41093CD057AF}</x14:id>
+          <x14:id>{FF96DA64-3300-434E-A209-C249AC9F0B17}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0C5285DE-770C-4BA1-B699-FB1D33570C86}</x14:id>
+          <x14:id>{A0C1FC2A-A972-40D5-BE6A-1364B0DA6D94}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{44C26EEA-516F-4C9A-86A5-53AE2A2A8895}</x14:id>
+          <x14:id>{8219CCB1-B4BA-4600-B581-DC74F5226F49}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DC79E82F-C20D-4114-B449-C25DC7EF690A}">
+          <x14:cfRule type="dataBar" id="{839CA61E-1EE3-405E-A487-E68717692F37}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9E082B04-E31F-46EB-89B0-41093CD057AF}">
+          <x14:cfRule type="dataBar" id="{FF96DA64-3300-434E-A209-C249AC9F0B17}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0C5285DE-770C-4BA1-B699-FB1D33570C86}">
+          <x14:cfRule type="dataBar" id="{A0C1FC2A-A972-40D5-BE6A-1364B0DA6D94}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{44C26EEA-516F-4C9A-86A5-53AE2A2A8895}">
+          <x14:cfRule type="dataBar" id="{8219CCB1-B4BA-4600-B581-DC74F5226F49}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6DCD2F68-D2C5-40AA-85E7-192FE793A81C}</x14:id>
+          <x14:id>{0D8B0E1B-7FB4-47F9-BD4C-35947194222C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A9B315FE-6419-406D-A826-4D5E1A4CBB4E}</x14:id>
+          <x14:id>{B5641BCB-323C-4B3F-96AF-A52013E397B9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7514BC41-566E-4EBC-BC4B-7A7CD1F0933A}</x14:id>
+          <x14:id>{FF013BA2-45D7-46E9-97B0-DC5ACB7C3408}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DA219EC9-98F7-4F3E-AD66-A6EFC67A3121}</x14:id>
+          <x14:id>{77CDC43A-5352-4139-8BE6-93394EEA4150}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6DCD2F68-D2C5-40AA-85E7-192FE793A81C}">
+          <x14:cfRule type="dataBar" id="{0D8B0E1B-7FB4-47F9-BD4C-35947194222C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A9B315FE-6419-406D-A826-4D5E1A4CBB4E}">
+          <x14:cfRule type="dataBar" id="{B5641BCB-323C-4B3F-96AF-A52013E397B9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7514BC41-566E-4EBC-BC4B-7A7CD1F0933A}">
+          <x14:cfRule type="dataBar" id="{FF013BA2-45D7-46E9-97B0-DC5ACB7C3408}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DA219EC9-98F7-4F3E-AD66-A6EFC67A3121}">
+          <x14:cfRule type="dataBar" id="{77CDC43A-5352-4139-8BE6-93394EEA4150}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{839CA61E-1EE3-405E-A487-E68717692F37}</x14:id>
+          <x14:id>{96250825-08EC-4E60-97DE-326955FA91A9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FF96DA64-3300-434E-A209-C249AC9F0B17}</x14:id>
+          <x14:id>{96C30BC1-B84D-41DE-96C8-A7B569C7C25B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A0C1FC2A-A972-40D5-BE6A-1364B0DA6D94}</x14:id>
+          <x14:id>{99C65F6A-3BFF-453F-B0AD-352939F771D4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8219CCB1-B4BA-4600-B581-DC74F5226F49}</x14:id>
+          <x14:id>{4050FA51-607C-4076-808E-FCD484F6E155}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{839CA61E-1EE3-405E-A487-E68717692F37}">
+          <x14:cfRule type="dataBar" id="{96250825-08EC-4E60-97DE-326955FA91A9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FF96DA64-3300-434E-A209-C249AC9F0B17}">
+          <x14:cfRule type="dataBar" id="{96C30BC1-B84D-41DE-96C8-A7B569C7C25B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A0C1FC2A-A972-40D5-BE6A-1364B0DA6D94}">
+          <x14:cfRule type="dataBar" id="{99C65F6A-3BFF-453F-B0AD-352939F771D4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8219CCB1-B4BA-4600-B581-DC74F5226F49}">
+          <x14:cfRule type="dataBar" id="{4050FA51-607C-4076-808E-FCD484F6E155}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0D8B0E1B-7FB4-47F9-BD4C-35947194222C}</x14:id>
+          <x14:id>{18A9FF47-8BB6-44C7-A4A8-75F2C14ECC6B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B5641BCB-323C-4B3F-96AF-A52013E397B9}</x14:id>
+          <x14:id>{B9507D60-43A8-4350-AA12-017AE705FD54}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FF013BA2-45D7-46E9-97B0-DC5ACB7C3408}</x14:id>
+          <x14:id>{EEC64ADB-EA42-49FD-A1EB-D313E1134326}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{77CDC43A-5352-4139-8BE6-93394EEA4150}</x14:id>
+          <x14:id>{AE38A89C-9556-4412-AB61-F43B2B283C45}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0D8B0E1B-7FB4-47F9-BD4C-35947194222C}">
+          <x14:cfRule type="dataBar" id="{18A9FF47-8BB6-44C7-A4A8-75F2C14ECC6B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B5641BCB-323C-4B3F-96AF-A52013E397B9}">
+          <x14:cfRule type="dataBar" id="{B9507D60-43A8-4350-AA12-017AE705FD54}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FF013BA2-45D7-46E9-97B0-DC5ACB7C3408}">
+          <x14:cfRule type="dataBar" id="{EEC64ADB-EA42-49FD-A1EB-D313E1134326}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{77CDC43A-5352-4139-8BE6-93394EEA4150}">
+          <x14:cfRule type="dataBar" id="{AE38A89C-9556-4412-AB61-F43B2B283C45}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{96250825-08EC-4E60-97DE-326955FA91A9}</x14:id>
+          <x14:id>{2694F18E-4E2A-4875-9048-FFBD2A77782F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{96C30BC1-B84D-41DE-96C8-A7B569C7C25B}</x14:id>
+          <x14:id>{D927876D-BA9C-4C71-A654-91EF60643803}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{99C65F6A-3BFF-453F-B0AD-352939F771D4}</x14:id>
+          <x14:id>{57ED4AB6-6217-421A-AB1A-E3CE13D6000A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4050FA51-607C-4076-808E-FCD484F6E155}</x14:id>
+          <x14:id>{8E84B391-1DB9-4B4F-A981-329F3979E613}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{96250825-08EC-4E60-97DE-326955FA91A9}">
+          <x14:cfRule type="dataBar" id="{2694F18E-4E2A-4875-9048-FFBD2A77782F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{96C30BC1-B84D-41DE-96C8-A7B569C7C25B}">
+          <x14:cfRule type="dataBar" id="{D927876D-BA9C-4C71-A654-91EF60643803}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{99C65F6A-3BFF-453F-B0AD-352939F771D4}">
+          <x14:cfRule type="dataBar" id="{57ED4AB6-6217-421A-AB1A-E3CE13D6000A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4050FA51-607C-4076-808E-FCD484F6E155}">
+          <x14:cfRule type="dataBar" id="{8E84B391-1DB9-4B4F-A981-329F3979E613}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{18A9FF47-8BB6-44C7-A4A8-75F2C14ECC6B}</x14:id>
+          <x14:id>{BE5EC536-E8BB-47AD-B2DB-FC82EDD1E933}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B9507D60-43A8-4350-AA12-017AE705FD54}</x14:id>
+          <x14:id>{7F64FE89-0592-4560-8E15-29BA634D32AA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EEC64ADB-EA42-49FD-A1EB-D313E1134326}</x14:id>
+          <x14:id>{CC123380-206F-4B31-A67F-3E1E6EE978B9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AE38A89C-9556-4412-AB61-F43B2B283C45}</x14:id>
+          <x14:id>{0DBA1D7E-247C-4658-95A7-848F7E8923FC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{18A9FF47-8BB6-44C7-A4A8-75F2C14ECC6B}">
+          <x14:cfRule type="dataBar" id="{BE5EC536-E8BB-47AD-B2DB-FC82EDD1E933}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B9507D60-43A8-4350-AA12-017AE705FD54}">
+          <x14:cfRule type="dataBar" id="{7F64FE89-0592-4560-8E15-29BA634D32AA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EEC64ADB-EA42-49FD-A1EB-D313E1134326}">
+          <x14:cfRule type="dataBar" id="{CC123380-206F-4B31-A67F-3E1E6EE978B9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AE38A89C-9556-4412-AB61-F43B2B283C45}">
+          <x14:cfRule type="dataBar" id="{0DBA1D7E-247C-4658-95A7-848F7E8923FC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2694F18E-4E2A-4875-9048-FFBD2A77782F}</x14:id>
+          <x14:id>{DCC30B73-47BC-4D2C-96F4-AB13AC76BC49}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D927876D-BA9C-4C71-A654-91EF60643803}</x14:id>
+          <x14:id>{055D1ACE-B4F5-4405-BD58-45F5552C7905}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{57ED4AB6-6217-421A-AB1A-E3CE13D6000A}</x14:id>
+          <x14:id>{926B7CB1-D0E5-444A-80EC-39C13306CB17}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8E84B391-1DB9-4B4F-A981-329F3979E613}</x14:id>
+          <x14:id>{A1B56C02-888D-4116-9486-B1DD11066359}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2694F18E-4E2A-4875-9048-FFBD2A77782F}">
+          <x14:cfRule type="dataBar" id="{DCC30B73-47BC-4D2C-96F4-AB13AC76BC49}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D927876D-BA9C-4C71-A654-91EF60643803}">
+          <x14:cfRule type="dataBar" id="{055D1ACE-B4F5-4405-BD58-45F5552C7905}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{57ED4AB6-6217-421A-AB1A-E3CE13D6000A}">
+          <x14:cfRule type="dataBar" id="{926B7CB1-D0E5-444A-80EC-39C13306CB17}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8E84B391-1DB9-4B4F-A981-329F3979E613}">
+          <x14:cfRule type="dataBar" id="{A1B56C02-888D-4116-9486-B1DD11066359}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BE5EC536-E8BB-47AD-B2DB-FC82EDD1E933}</x14:id>
+          <x14:id>{20AB7E0B-D17C-4F6E-AA23-9F98E2C8001F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F64FE89-0592-4560-8E15-29BA634D32AA}</x14:id>
+          <x14:id>{8A4C75CA-846F-4802-A4D5-056A87B63B24}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CC123380-206F-4B31-A67F-3E1E6EE978B9}</x14:id>
+          <x14:id>{BFDE5C18-99CB-4163-9E31-676E542E6527}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0DBA1D7E-247C-4658-95A7-848F7E8923FC}</x14:id>
+          <x14:id>{2E50AFB8-BBF9-4785-946D-BD8A60D046EE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BE5EC536-E8BB-47AD-B2DB-FC82EDD1E933}">
+          <x14:cfRule type="dataBar" id="{20AB7E0B-D17C-4F6E-AA23-9F98E2C8001F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F64FE89-0592-4560-8E15-29BA634D32AA}">
+          <x14:cfRule type="dataBar" id="{8A4C75CA-846F-4802-A4D5-056A87B63B24}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CC123380-206F-4B31-A67F-3E1E6EE978B9}">
+          <x14:cfRule type="dataBar" id="{BFDE5C18-99CB-4163-9E31-676E542E6527}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0DBA1D7E-247C-4658-95A7-848F7E8923FC}">
+          <x14:cfRule type="dataBar" id="{2E50AFB8-BBF9-4785-946D-BD8A60D046EE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DCC30B73-47BC-4D2C-96F4-AB13AC76BC49}</x14:id>
+          <x14:id>{42B1AA04-77D7-4B8F-B3D5-B08A63D14E85}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{055D1ACE-B4F5-4405-BD58-45F5552C7905}</x14:id>
+          <x14:id>{74B47D19-5DAC-4E37-BC52-E92E81566ED4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{926B7CB1-D0E5-444A-80EC-39C13306CB17}</x14:id>
+          <x14:id>{B96BC06E-6A1A-47E4-AF07-A6034E512AD9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A1B56C02-888D-4116-9486-B1DD11066359}</x14:id>
+          <x14:id>{21DF6B78-D419-4976-9866-D8610117390A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DCC30B73-47BC-4D2C-96F4-AB13AC76BC49}">
+          <x14:cfRule type="dataBar" id="{42B1AA04-77D7-4B8F-B3D5-B08A63D14E85}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{055D1ACE-B4F5-4405-BD58-45F5552C7905}">
+          <x14:cfRule type="dataBar" id="{74B47D19-5DAC-4E37-BC52-E92E81566ED4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{926B7CB1-D0E5-444A-80EC-39C13306CB17}">
+          <x14:cfRule type="dataBar" id="{B96BC06E-6A1A-47E4-AF07-A6034E512AD9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A1B56C02-888D-4116-9486-B1DD11066359}">
+          <x14:cfRule type="dataBar" id="{21DF6B78-D419-4976-9866-D8610117390A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{20AB7E0B-D17C-4F6E-AA23-9F98E2C8001F}</x14:id>
+          <x14:id>{F2DB8A46-2183-4A07-B3D0-AABA34E04542}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8A4C75CA-846F-4802-A4D5-056A87B63B24}</x14:id>
+          <x14:id>{4B6E0DAE-F998-4FBA-8514-11CB9A95ACD7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BFDE5C18-99CB-4163-9E31-676E542E6527}</x14:id>
+          <x14:id>{65F8CDCE-43FC-4B35-99A8-07155D4EDFE9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2E50AFB8-BBF9-4785-946D-BD8A60D046EE}</x14:id>
+          <x14:id>{71B7BB7A-A02B-4FE5-9BC6-1489B037B7FC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{20AB7E0B-D17C-4F6E-AA23-9F98E2C8001F}">
+          <x14:cfRule type="dataBar" id="{F2DB8A46-2183-4A07-B3D0-AABA34E04542}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8A4C75CA-846F-4802-A4D5-056A87B63B24}">
+          <x14:cfRule type="dataBar" id="{4B6E0DAE-F998-4FBA-8514-11CB9A95ACD7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BFDE5C18-99CB-4163-9E31-676E542E6527}">
+          <x14:cfRule type="dataBar" id="{65F8CDCE-43FC-4B35-99A8-07155D4EDFE9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2E50AFB8-BBF9-4785-946D-BD8A60D046EE}">
+          <x14:cfRule type="dataBar" id="{71B7BB7A-A02B-4FE5-9BC6-1489B037B7FC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{42B1AA04-77D7-4B8F-B3D5-B08A63D14E85}</x14:id>
+          <x14:id>{EC677F52-0129-43D0-AE74-2777A722661A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{74B47D19-5DAC-4E37-BC52-E92E81566ED4}</x14:id>
+          <x14:id>{C5B521F7-3D83-419C-AE4E-8EC68CBC5002}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B96BC06E-6A1A-47E4-AF07-A6034E512AD9}</x14:id>
+          <x14:id>{9F446DCA-F7EA-44E0-AAD4-9DD015AD1240}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{21DF6B78-D419-4976-9866-D8610117390A}</x14:id>
+          <x14:id>{AF5CE8DD-A0D8-4B7A-8A22-7E6669734BA2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{42B1AA04-77D7-4B8F-B3D5-B08A63D14E85}">
+          <x14:cfRule type="dataBar" id="{EC677F52-0129-43D0-AE74-2777A722661A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{74B47D19-5DAC-4E37-BC52-E92E81566ED4}">
+          <x14:cfRule type="dataBar" id="{C5B521F7-3D83-419C-AE4E-8EC68CBC5002}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B96BC06E-6A1A-47E4-AF07-A6034E512AD9}">
+          <x14:cfRule type="dataBar" id="{9F446DCA-F7EA-44E0-AAD4-9DD015AD1240}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{21DF6B78-D419-4976-9866-D8610117390A}">
+          <x14:cfRule type="dataBar" id="{AF5CE8DD-A0D8-4B7A-8A22-7E6669734BA2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F2DB8A46-2183-4A07-B3D0-AABA34E04542}</x14:id>
+          <x14:id>{FC144E2D-FF35-426F-9911-0E946AF5F1D6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4B6E0DAE-F998-4FBA-8514-11CB9A95ACD7}</x14:id>
+          <x14:id>{35ACC8D0-60C1-43F8-8D46-3830005E0D4F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{65F8CDCE-43FC-4B35-99A8-07155D4EDFE9}</x14:id>
+          <x14:id>{1A795798-C9BD-47B0-A4A8-5E4FADD05CA3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{71B7BB7A-A02B-4FE5-9BC6-1489B037B7FC}</x14:id>
+          <x14:id>{508C5A17-0DD3-480A-8376-BA05A2943009}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F2DB8A46-2183-4A07-B3D0-AABA34E04542}">
+          <x14:cfRule type="dataBar" id="{FC144E2D-FF35-426F-9911-0E946AF5F1D6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4B6E0DAE-F998-4FBA-8514-11CB9A95ACD7}">
+          <x14:cfRule type="dataBar" id="{35ACC8D0-60C1-43F8-8D46-3830005E0D4F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{65F8CDCE-43FC-4B35-99A8-07155D4EDFE9}">
+          <x14:cfRule type="dataBar" id="{1A795798-C9BD-47B0-A4A8-5E4FADD05CA3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{71B7BB7A-A02B-4FE5-9BC6-1489B037B7FC}">
+          <x14:cfRule type="dataBar" id="{508C5A17-0DD3-480A-8376-BA05A2943009}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EC677F52-0129-43D0-AE74-2777A722661A}</x14:id>
+          <x14:id>{DF0ED3AC-5103-4FE7-8119-A944B0C8F0A7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C5B521F7-3D83-419C-AE4E-8EC68CBC5002}</x14:id>
+          <x14:id>{2FC9AA6B-6DB9-424A-9DC7-054DDCCC790F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9F446DCA-F7EA-44E0-AAD4-9DD015AD1240}</x14:id>
+          <x14:id>{E86CCB73-1CE7-48A0-AC39-76659E2282B4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AF5CE8DD-A0D8-4B7A-8A22-7E6669734BA2}</x14:id>
+          <x14:id>{414538CC-9563-4446-A857-F79A8B69391D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EC677F52-0129-43D0-AE74-2777A722661A}">
+          <x14:cfRule type="dataBar" id="{DF0ED3AC-5103-4FE7-8119-A944B0C8F0A7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C5B521F7-3D83-419C-AE4E-8EC68CBC5002}">
+          <x14:cfRule type="dataBar" id="{2FC9AA6B-6DB9-424A-9DC7-054DDCCC790F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9F446DCA-F7EA-44E0-AAD4-9DD015AD1240}">
+          <x14:cfRule type="dataBar" id="{E86CCB73-1CE7-48A0-AC39-76659E2282B4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AF5CE8DD-A0D8-4B7A-8A22-7E6669734BA2}">
+          <x14:cfRule type="dataBar" id="{414538CC-9563-4446-A857-F79A8B69391D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FC144E2D-FF35-426F-9911-0E946AF5F1D6}</x14:id>
+          <x14:id>{A0C1807A-2FA8-46FF-A3AB-BE96DA4E7A25}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{35ACC8D0-60C1-43F8-8D46-3830005E0D4F}</x14:id>
+          <x14:id>{7E9682AC-0D73-4F87-88B5-3F069609388B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1A795798-C9BD-47B0-A4A8-5E4FADD05CA3}</x14:id>
+          <x14:id>{45D45710-47F6-4365-BBC8-FF6477F94AE3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{508C5A17-0DD3-480A-8376-BA05A2943009}</x14:id>
+          <x14:id>{38BF6850-88EF-4BA5-A522-1906991A77B7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FC144E2D-FF35-426F-9911-0E946AF5F1D6}">
+          <x14:cfRule type="dataBar" id="{A0C1807A-2FA8-46FF-A3AB-BE96DA4E7A25}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{35ACC8D0-60C1-43F8-8D46-3830005E0D4F}">
+          <x14:cfRule type="dataBar" id="{7E9682AC-0D73-4F87-88B5-3F069609388B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1A795798-C9BD-47B0-A4A8-5E4FADD05CA3}">
+          <x14:cfRule type="dataBar" id="{45D45710-47F6-4365-BBC8-FF6477F94AE3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{508C5A17-0DD3-480A-8376-BA05A2943009}">
+          <x14:cfRule type="dataBar" id="{38BF6850-88EF-4BA5-A522-1906991A77B7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-15 09:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -11225,7 +11225,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DF0ED3AC-5103-4FE7-8119-A944B0C8F0A7}</x14:id>
+          <x14:id>{3B96CE5A-12F9-4463-9DD2-485029C48963}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11239,7 +11239,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2FC9AA6B-6DB9-424A-9DC7-054DDCCC790F}</x14:id>
+          <x14:id>{B3F42A2E-B906-4F5E-AE71-0B7539233DDF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11253,7 +11253,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E86CCB73-1CE7-48A0-AC39-76659E2282B4}</x14:id>
+          <x14:id>{FC3D19C0-77B2-4541-8667-8CBA8F616608}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11267,7 +11267,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{414538CC-9563-4446-A857-F79A8B69391D}</x14:id>
+          <x14:id>{1E10DAFF-3B7A-430C-9032-0D045149B3B0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11277,7 +11277,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DF0ED3AC-5103-4FE7-8119-A944B0C8F0A7}">
+          <x14:cfRule type="dataBar" id="{3B96CE5A-12F9-4463-9DD2-485029C48963}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11290,7 +11290,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2FC9AA6B-6DB9-424A-9DC7-054DDCCC790F}">
+          <x14:cfRule type="dataBar" id="{B3F42A2E-B906-4F5E-AE71-0B7539233DDF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11303,7 +11303,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E86CCB73-1CE7-48A0-AC39-76659E2282B4}">
+          <x14:cfRule type="dataBar" id="{FC3D19C0-77B2-4541-8667-8CBA8F616608}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11316,7 +11316,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{414538CC-9563-4446-A857-F79A8B69391D}">
+          <x14:cfRule type="dataBar" id="{1E10DAFF-3B7A-430C-9032-0D045149B3B0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26961,7 +26961,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A0C1807A-2FA8-46FF-A3AB-BE96DA4E7A25}</x14:id>
+          <x14:id>{3A637B0A-3913-4FBD-AA8A-267004FD3011}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26975,7 +26975,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7E9682AC-0D73-4F87-88B5-3F069609388B}</x14:id>
+          <x14:id>{16D90FF6-EFA8-4D8A-9954-AF3181A849D3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26989,7 +26989,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{45D45710-47F6-4365-BBC8-FF6477F94AE3}</x14:id>
+          <x14:id>{501B339A-3F92-49D8-B30B-35BAA137C7BF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27003,7 +27003,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{38BF6850-88EF-4BA5-A522-1906991A77B7}</x14:id>
+          <x14:id>{EDFDB890-EA9B-4C76-ADF9-6F1895F84E2A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27013,7 +27013,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A0C1807A-2FA8-46FF-A3AB-BE96DA4E7A25}">
+          <x14:cfRule type="dataBar" id="{3A637B0A-3913-4FBD-AA8A-267004FD3011}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27026,7 +27026,7 @@
           <xm:sqref>N6:N176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7E9682AC-0D73-4F87-88B5-3F069609388B}">
+          <x14:cfRule type="dataBar" id="{16D90FF6-EFA8-4D8A-9954-AF3181A849D3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27039,7 +27039,7 @@
           <xm:sqref>P6:P176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{45D45710-47F6-4365-BBC8-FF6477F94AE3}">
+          <x14:cfRule type="dataBar" id="{501B339A-3F92-49D8-B30B-35BAA137C7BF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27052,7 +27052,7 @@
           <xm:sqref>Y6:Y176</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{38BF6850-88EF-4BA5-A522-1906991A77B7}">
+          <x14:cfRule type="dataBar" id="{EDFDB890-EA9B-4C76-ADF9-6F1895F84E2A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 07:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C9EADDFB-C11A-4EE7-AA36-198F68305B70}</x14:id>
+          <x14:id>{DA3452F2-9881-42C7-BAD2-EC700B081AFE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1A21194F-962B-46A7-80FB-572558C15F93}</x14:id>
+          <x14:id>{5DEB0920-E822-4948-9BAD-BF19C926FA5F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A8E11B03-CF69-41D9-AEC5-A0C55368F4B8}</x14:id>
+          <x14:id>{DD4964D0-D547-43E3-9903-1448491B8B76}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7FB6F097-1A28-4495-B38D-637B972742D2}</x14:id>
+          <x14:id>{B9356866-88FA-4BB2-81D7-55577BC1417D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C9EADDFB-C11A-4EE7-AA36-198F68305B70}">
+          <x14:cfRule type="dataBar" id="{DA3452F2-9881-42C7-BAD2-EC700B081AFE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1A21194F-962B-46A7-80FB-572558C15F93}">
+          <x14:cfRule type="dataBar" id="{5DEB0920-E822-4948-9BAD-BF19C926FA5F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A8E11B03-CF69-41D9-AEC5-A0C55368F4B8}">
+          <x14:cfRule type="dataBar" id="{DD4964D0-D547-43E3-9903-1448491B8B76}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7FB6F097-1A28-4495-B38D-637B972742D2}">
+          <x14:cfRule type="dataBar" id="{B9356866-88FA-4BB2-81D7-55577BC1417D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A126829F-9255-4DBB-A309-3F43957DB27A}</x14:id>
+          <x14:id>{B61EA627-654D-491F-B548-7CD86321F5EC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E45AB1F4-FBCA-4765-9259-57240AF74A59}</x14:id>
+          <x14:id>{6CA9C8E9-73A9-4AD1-8B08-8ABB620F2C50}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4B187DB6-4A44-4252-97D1-D4E1D8F1CBE8}</x14:id>
+          <x14:id>{38E3939B-BE9F-40DD-B3BA-E5CDD79A8C76}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A578B6A7-110E-4069-BBA1-862DC7943376}</x14:id>
+          <x14:id>{1E1E7375-90CE-484B-8DB5-E8C4648C17B7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A126829F-9255-4DBB-A309-3F43957DB27A}">
+          <x14:cfRule type="dataBar" id="{B61EA627-654D-491F-B548-7CD86321F5EC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E45AB1F4-FBCA-4765-9259-57240AF74A59}">
+          <x14:cfRule type="dataBar" id="{6CA9C8E9-73A9-4AD1-8B08-8ABB620F2C50}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4B187DB6-4A44-4252-97D1-D4E1D8F1CBE8}">
+          <x14:cfRule type="dataBar" id="{38E3939B-BE9F-40DD-B3BA-E5CDD79A8C76}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A578B6A7-110E-4069-BBA1-862DC7943376}">
+          <x14:cfRule type="dataBar" id="{1E1E7375-90CE-484B-8DB5-E8C4648C17B7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DA3452F2-9881-42C7-BAD2-EC700B081AFE}</x14:id>
+          <x14:id>{C66E88A8-AA44-4896-B74C-8B184AFCC55B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5DEB0920-E822-4948-9BAD-BF19C926FA5F}</x14:id>
+          <x14:id>{99F9F078-D1B5-462A-AF83-7CC81D9D6143}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DD4964D0-D547-43E3-9903-1448491B8B76}</x14:id>
+          <x14:id>{9FD2C364-6324-422A-8845-624A7F1F745A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B9356866-88FA-4BB2-81D7-55577BC1417D}</x14:id>
+          <x14:id>{1CABB76E-7962-48AD-B56E-03F44F881903}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DA3452F2-9881-42C7-BAD2-EC700B081AFE}">
+          <x14:cfRule type="dataBar" id="{C66E88A8-AA44-4896-B74C-8B184AFCC55B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5DEB0920-E822-4948-9BAD-BF19C926FA5F}">
+          <x14:cfRule type="dataBar" id="{99F9F078-D1B5-462A-AF83-7CC81D9D6143}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DD4964D0-D547-43E3-9903-1448491B8B76}">
+          <x14:cfRule type="dataBar" id="{9FD2C364-6324-422A-8845-624A7F1F745A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B9356866-88FA-4BB2-81D7-55577BC1417D}">
+          <x14:cfRule type="dataBar" id="{1CABB76E-7962-48AD-B56E-03F44F881903}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B61EA627-654D-491F-B548-7CD86321F5EC}</x14:id>
+          <x14:id>{DA1359C2-6B8E-43C1-842E-B104D16F68A0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6CA9C8E9-73A9-4AD1-8B08-8ABB620F2C50}</x14:id>
+          <x14:id>{AA9CE8A9-70FC-4213-940C-69CBC0906872}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{38E3939B-BE9F-40DD-B3BA-E5CDD79A8C76}</x14:id>
+          <x14:id>{451DA441-112D-49BE-A679-E5CEA9294BC2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1E1E7375-90CE-484B-8DB5-E8C4648C17B7}</x14:id>
+          <x14:id>{858AF25E-6623-440B-9EEC-824F68D26D3E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B61EA627-654D-491F-B548-7CD86321F5EC}">
+          <x14:cfRule type="dataBar" id="{DA1359C2-6B8E-43C1-842E-B104D16F68A0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6CA9C8E9-73A9-4AD1-8B08-8ABB620F2C50}">
+          <x14:cfRule type="dataBar" id="{AA9CE8A9-70FC-4213-940C-69CBC0906872}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{38E3939B-BE9F-40DD-B3BA-E5CDD79A8C76}">
+          <x14:cfRule type="dataBar" id="{451DA441-112D-49BE-A679-E5CEA9294BC2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1E1E7375-90CE-484B-8DB5-E8C4648C17B7}">
+          <x14:cfRule type="dataBar" id="{858AF25E-6623-440B-9EEC-824F68D26D3E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C66E88A8-AA44-4896-B74C-8B184AFCC55B}</x14:id>
+          <x14:id>{756F3B45-E2F3-401D-9E38-3FCCBDA37950}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{99F9F078-D1B5-462A-AF83-7CC81D9D6143}</x14:id>
+          <x14:id>{5A197A4B-9F05-4311-B5DD-A036CF190393}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9FD2C364-6324-422A-8845-624A7F1F745A}</x14:id>
+          <x14:id>{169752D0-2A90-4B6C-B29E-53E62A804560}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1CABB76E-7962-48AD-B56E-03F44F881903}</x14:id>
+          <x14:id>{6A4F8798-E637-4F11-A6DA-B8C82D845ECD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C66E88A8-AA44-4896-B74C-8B184AFCC55B}">
+          <x14:cfRule type="dataBar" id="{756F3B45-E2F3-401D-9E38-3FCCBDA37950}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{99F9F078-D1B5-462A-AF83-7CC81D9D6143}">
+          <x14:cfRule type="dataBar" id="{5A197A4B-9F05-4311-B5DD-A036CF190393}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9FD2C364-6324-422A-8845-624A7F1F745A}">
+          <x14:cfRule type="dataBar" id="{169752D0-2A90-4B6C-B29E-53E62A804560}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1CABB76E-7962-48AD-B56E-03F44F881903}">
+          <x14:cfRule type="dataBar" id="{6A4F8798-E637-4F11-A6DA-B8C82D845ECD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DA1359C2-6B8E-43C1-842E-B104D16F68A0}</x14:id>
+          <x14:id>{252F812E-0E04-4F9E-B077-55D114073253}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AA9CE8A9-70FC-4213-940C-69CBC0906872}</x14:id>
+          <x14:id>{C1EA4FEA-31B7-4750-8754-5F92317F20F5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{451DA441-112D-49BE-A679-E5CEA9294BC2}</x14:id>
+          <x14:id>{F0C9F420-2FD8-4FE6-A7C0-0D88979ADA09}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{858AF25E-6623-440B-9EEC-824F68D26D3E}</x14:id>
+          <x14:id>{D8D28FFC-8108-4278-8DEC-84079E381E02}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DA1359C2-6B8E-43C1-842E-B104D16F68A0}">
+          <x14:cfRule type="dataBar" id="{252F812E-0E04-4F9E-B077-55D114073253}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AA9CE8A9-70FC-4213-940C-69CBC0906872}">
+          <x14:cfRule type="dataBar" id="{C1EA4FEA-31B7-4750-8754-5F92317F20F5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{451DA441-112D-49BE-A679-E5CEA9294BC2}">
+          <x14:cfRule type="dataBar" id="{F0C9F420-2FD8-4FE6-A7C0-0D88979ADA09}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{858AF25E-6623-440B-9EEC-824F68D26D3E}">
+          <x14:cfRule type="dataBar" id="{D8D28FFC-8108-4278-8DEC-84079E381E02}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{756F3B45-E2F3-401D-9E38-3FCCBDA37950}</x14:id>
+          <x14:id>{44980546-1497-4DAE-BB1A-4526B844F04F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5A197A4B-9F05-4311-B5DD-A036CF190393}</x14:id>
+          <x14:id>{C2E62083-48E1-4662-8CFA-19C70B1693B5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{169752D0-2A90-4B6C-B29E-53E62A804560}</x14:id>
+          <x14:id>{0914170B-FAFA-4358-A873-375B1009E6A3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6A4F8798-E637-4F11-A6DA-B8C82D845ECD}</x14:id>
+          <x14:id>{A0BE8092-D24E-47F1-A72B-94CCD0D9F775}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{756F3B45-E2F3-401D-9E38-3FCCBDA37950}">
+          <x14:cfRule type="dataBar" id="{44980546-1497-4DAE-BB1A-4526B844F04F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5A197A4B-9F05-4311-B5DD-A036CF190393}">
+          <x14:cfRule type="dataBar" id="{C2E62083-48E1-4662-8CFA-19C70B1693B5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{169752D0-2A90-4B6C-B29E-53E62A804560}">
+          <x14:cfRule type="dataBar" id="{0914170B-FAFA-4358-A873-375B1009E6A3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6A4F8798-E637-4F11-A6DA-B8C82D845ECD}">
+          <x14:cfRule type="dataBar" id="{A0BE8092-D24E-47F1-A72B-94CCD0D9F775}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{252F812E-0E04-4F9E-B077-55D114073253}</x14:id>
+          <x14:id>{9842537F-FB37-4D6A-91DB-2478794A6BA4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C1EA4FEA-31B7-4750-8754-5F92317F20F5}</x14:id>
+          <x14:id>{450903E6-358B-4D48-BD77-07330557CF06}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F0C9F420-2FD8-4FE6-A7C0-0D88979ADA09}</x14:id>
+          <x14:id>{2120E51B-B0CC-40D3-96FD-A1BE74275D3F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D8D28FFC-8108-4278-8DEC-84079E381E02}</x14:id>
+          <x14:id>{6B5CA8CE-4BDD-4270-BDCB-70B8DA8CAFB5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{252F812E-0E04-4F9E-B077-55D114073253}">
+          <x14:cfRule type="dataBar" id="{9842537F-FB37-4D6A-91DB-2478794A6BA4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C1EA4FEA-31B7-4750-8754-5F92317F20F5}">
+          <x14:cfRule type="dataBar" id="{450903E6-358B-4D48-BD77-07330557CF06}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F0C9F420-2FD8-4FE6-A7C0-0D88979ADA09}">
+          <x14:cfRule type="dataBar" id="{2120E51B-B0CC-40D3-96FD-A1BE74275D3F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D8D28FFC-8108-4278-8DEC-84079E381E02}">
+          <x14:cfRule type="dataBar" id="{6B5CA8CE-4BDD-4270-BDCB-70B8DA8CAFB5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{44980546-1497-4DAE-BB1A-4526B844F04F}</x14:id>
+          <x14:id>{FBE7D80F-4BD1-4C11-A8F6-81544389D0EC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C2E62083-48E1-4662-8CFA-19C70B1693B5}</x14:id>
+          <x14:id>{7A272AD5-CE4D-4A83-8D21-69A5043D0BE7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0914170B-FAFA-4358-A873-375B1009E6A3}</x14:id>
+          <x14:id>{2FBFE501-D5CB-4869-A270-D95B3AA15E3F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A0BE8092-D24E-47F1-A72B-94CCD0D9F775}</x14:id>
+          <x14:id>{E9FBBBF1-53F7-4E6A-8578-BA1631C8D0AC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{44980546-1497-4DAE-BB1A-4526B844F04F}">
+          <x14:cfRule type="dataBar" id="{FBE7D80F-4BD1-4C11-A8F6-81544389D0EC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C2E62083-48E1-4662-8CFA-19C70B1693B5}">
+          <x14:cfRule type="dataBar" id="{7A272AD5-CE4D-4A83-8D21-69A5043D0BE7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0914170B-FAFA-4358-A873-375B1009E6A3}">
+          <x14:cfRule type="dataBar" id="{2FBFE501-D5CB-4869-A270-D95B3AA15E3F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A0BE8092-D24E-47F1-A72B-94CCD0D9F775}">
+          <x14:cfRule type="dataBar" id="{E9FBBBF1-53F7-4E6A-8578-BA1631C8D0AC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9842537F-FB37-4D6A-91DB-2478794A6BA4}</x14:id>
+          <x14:id>{5D61A293-645A-484B-863F-7E33C6FB3140}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{450903E6-358B-4D48-BD77-07330557CF06}</x14:id>
+          <x14:id>{4BA254F9-3779-4FBF-9E27-18346CEC4096}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2120E51B-B0CC-40D3-96FD-A1BE74275D3F}</x14:id>
+          <x14:id>{78456BED-7AC4-464A-AF6C-B816D01FDC67}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6B5CA8CE-4BDD-4270-BDCB-70B8DA8CAFB5}</x14:id>
+          <x14:id>{2B69510A-45AD-43F7-A033-858B02E62754}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9842537F-FB37-4D6A-91DB-2478794A6BA4}">
+          <x14:cfRule type="dataBar" id="{5D61A293-645A-484B-863F-7E33C6FB3140}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{450903E6-358B-4D48-BD77-07330557CF06}">
+          <x14:cfRule type="dataBar" id="{4BA254F9-3779-4FBF-9E27-18346CEC4096}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2120E51B-B0CC-40D3-96FD-A1BE74275D3F}">
+          <x14:cfRule type="dataBar" id="{78456BED-7AC4-464A-AF6C-B816D01FDC67}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6B5CA8CE-4BDD-4270-BDCB-70B8DA8CAFB5}">
+          <x14:cfRule type="dataBar" id="{2B69510A-45AD-43F7-A033-858B02E62754}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FBE7D80F-4BD1-4C11-A8F6-81544389D0EC}</x14:id>
+          <x14:id>{97CBA6EF-B7DB-4E68-AA91-9380B244EEB7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7A272AD5-CE4D-4A83-8D21-69A5043D0BE7}</x14:id>
+          <x14:id>{7557162A-0D18-4900-B352-B4C390333CF6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2FBFE501-D5CB-4869-A270-D95B3AA15E3F}</x14:id>
+          <x14:id>{B96BF3DE-D539-4E55-AECB-C5C549625FE2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E9FBBBF1-53F7-4E6A-8578-BA1631C8D0AC}</x14:id>
+          <x14:id>{D2F944BD-0568-4273-8B5F-BD9B78410EE2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FBE7D80F-4BD1-4C11-A8F6-81544389D0EC}">
+          <x14:cfRule type="dataBar" id="{97CBA6EF-B7DB-4E68-AA91-9380B244EEB7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7A272AD5-CE4D-4A83-8D21-69A5043D0BE7}">
+          <x14:cfRule type="dataBar" id="{7557162A-0D18-4900-B352-B4C390333CF6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2FBFE501-D5CB-4869-A270-D95B3AA15E3F}">
+          <x14:cfRule type="dataBar" id="{B96BF3DE-D539-4E55-AECB-C5C549625FE2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E9FBBBF1-53F7-4E6A-8578-BA1631C8D0AC}">
+          <x14:cfRule type="dataBar" id="{D2F944BD-0568-4273-8B5F-BD9B78410EE2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5D61A293-645A-484B-863F-7E33C6FB3140}</x14:id>
+          <x14:id>{1414D308-0E36-4F7E-966C-31EE16F33A08}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4BA254F9-3779-4FBF-9E27-18346CEC4096}</x14:id>
+          <x14:id>{66E8AF0E-A934-4A8C-8B7A-45D19FBDD2F3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{78456BED-7AC4-464A-AF6C-B816D01FDC67}</x14:id>
+          <x14:id>{1977075C-B3F2-47D6-BDFA-94442DBC9296}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2B69510A-45AD-43F7-A033-858B02E62754}</x14:id>
+          <x14:id>{2D5A50C6-3A7A-4A90-AEDC-EB8A1740F8FD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5D61A293-645A-484B-863F-7E33C6FB3140}">
+          <x14:cfRule type="dataBar" id="{1414D308-0E36-4F7E-966C-31EE16F33A08}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4BA254F9-3779-4FBF-9E27-18346CEC4096}">
+          <x14:cfRule type="dataBar" id="{66E8AF0E-A934-4A8C-8B7A-45D19FBDD2F3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{78456BED-7AC4-464A-AF6C-B816D01FDC67}">
+          <x14:cfRule type="dataBar" id="{1977075C-B3F2-47D6-BDFA-94442DBC9296}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2B69510A-45AD-43F7-A033-858B02E62754}">
+          <x14:cfRule type="dataBar" id="{2D5A50C6-3A7A-4A90-AEDC-EB8A1740F8FD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{97CBA6EF-B7DB-4E68-AA91-9380B244EEB7}</x14:id>
+          <x14:id>{17C56633-C6B1-45C3-B184-1B8134C86896}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7557162A-0D18-4900-B352-B4C390333CF6}</x14:id>
+          <x14:id>{9E77C883-288F-4991-B8B1-102E9B8B75B1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B96BF3DE-D539-4E55-AECB-C5C549625FE2}</x14:id>
+          <x14:id>{7596520F-AD52-4FB8-B12A-D97A3EB47956}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D2F944BD-0568-4273-8B5F-BD9B78410EE2}</x14:id>
+          <x14:id>{2D4A44C5-739A-4D5D-8608-A46ED5F751AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{97CBA6EF-B7DB-4E68-AA91-9380B244EEB7}">
+          <x14:cfRule type="dataBar" id="{17C56633-C6B1-45C3-B184-1B8134C86896}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7557162A-0D18-4900-B352-B4C390333CF6}">
+          <x14:cfRule type="dataBar" id="{9E77C883-288F-4991-B8B1-102E9B8B75B1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B96BF3DE-D539-4E55-AECB-C5C549625FE2}">
+          <x14:cfRule type="dataBar" id="{7596520F-AD52-4FB8-B12A-D97A3EB47956}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D2F944BD-0568-4273-8B5F-BD9B78410EE2}">
+          <x14:cfRule type="dataBar" id="{2D4A44C5-739A-4D5D-8608-A46ED5F751AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1414D308-0E36-4F7E-966C-31EE16F33A08}</x14:id>
+          <x14:id>{538281A1-81CC-4A01-BC5D-3988C73FBE86}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{66E8AF0E-A934-4A8C-8B7A-45D19FBDD2F3}</x14:id>
+          <x14:id>{288AACEA-20F9-4FBC-A2B5-B8E9D471C0AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1977075C-B3F2-47D6-BDFA-94442DBC9296}</x14:id>
+          <x14:id>{B6F33F4D-CC76-4C7C-9A55-9442CC4942F3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2D5A50C6-3A7A-4A90-AEDC-EB8A1740F8FD}</x14:id>
+          <x14:id>{DBCEC498-91A7-411D-A5F3-FB0DAE0646D6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1414D308-0E36-4F7E-966C-31EE16F33A08}">
+          <x14:cfRule type="dataBar" id="{538281A1-81CC-4A01-BC5D-3988C73FBE86}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{66E8AF0E-A934-4A8C-8B7A-45D19FBDD2F3}">
+          <x14:cfRule type="dataBar" id="{288AACEA-20F9-4FBC-A2B5-B8E9D471C0AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1977075C-B3F2-47D6-BDFA-94442DBC9296}">
+          <x14:cfRule type="dataBar" id="{B6F33F4D-CC76-4C7C-9A55-9442CC4942F3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2D5A50C6-3A7A-4A90-AEDC-EB8A1740F8FD}">
+          <x14:cfRule type="dataBar" id="{DBCEC498-91A7-411D-A5F3-FB0DAE0646D6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{17C56633-C6B1-45C3-B184-1B8134C86896}</x14:id>
+          <x14:id>{127C0B17-8994-45FA-8363-20555E55FD77}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9E77C883-288F-4991-B8B1-102E9B8B75B1}</x14:id>
+          <x14:id>{6AF82B66-A67E-4644-A5D9-09BA219ADA00}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7596520F-AD52-4FB8-B12A-D97A3EB47956}</x14:id>
+          <x14:id>{759CDCC4-A548-429E-974A-808A28EFB8FC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2D4A44C5-739A-4D5D-8608-A46ED5F751AB}</x14:id>
+          <x14:id>{D5B1C543-A861-44A8-80B4-85670AA1D666}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{17C56633-C6B1-45C3-B184-1B8134C86896}">
+          <x14:cfRule type="dataBar" id="{127C0B17-8994-45FA-8363-20555E55FD77}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9E77C883-288F-4991-B8B1-102E9B8B75B1}">
+          <x14:cfRule type="dataBar" id="{6AF82B66-A67E-4644-A5D9-09BA219ADA00}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7596520F-AD52-4FB8-B12A-D97A3EB47956}">
+          <x14:cfRule type="dataBar" id="{759CDCC4-A548-429E-974A-808A28EFB8FC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2D4A44C5-739A-4D5D-8608-A46ED5F751AB}">
+          <x14:cfRule type="dataBar" id="{D5B1C543-A861-44A8-80B4-85670AA1D666}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{538281A1-81CC-4A01-BC5D-3988C73FBE86}</x14:id>
+          <x14:id>{25D9CEDA-CD9F-4E46-8ED0-45C1A4303DCF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{288AACEA-20F9-4FBC-A2B5-B8E9D471C0AB}</x14:id>
+          <x14:id>{2AFE3761-29A1-4DC7-BC35-BAB65A532456}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B6F33F4D-CC76-4C7C-9A55-9442CC4942F3}</x14:id>
+          <x14:id>{484EF240-57E1-4DBE-8676-7E0E49569E5F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DBCEC498-91A7-411D-A5F3-FB0DAE0646D6}</x14:id>
+          <x14:id>{8C483254-A6E4-499A-AB4C-A642BF0493D1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{538281A1-81CC-4A01-BC5D-3988C73FBE86}">
+          <x14:cfRule type="dataBar" id="{25D9CEDA-CD9F-4E46-8ED0-45C1A4303DCF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{288AACEA-20F9-4FBC-A2B5-B8E9D471C0AB}">
+          <x14:cfRule type="dataBar" id="{2AFE3761-29A1-4DC7-BC35-BAB65A532456}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B6F33F4D-CC76-4C7C-9A55-9442CC4942F3}">
+          <x14:cfRule type="dataBar" id="{484EF240-57E1-4DBE-8676-7E0E49569E5F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DBCEC498-91A7-411D-A5F3-FB0DAE0646D6}">
+          <x14:cfRule type="dataBar" id="{8C483254-A6E4-499A-AB4C-A642BF0493D1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{127C0B17-8994-45FA-8363-20555E55FD77}</x14:id>
+          <x14:id>{0E3ABD57-7597-4A6F-A9CF-B218657A67B4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6AF82B66-A67E-4644-A5D9-09BA219ADA00}</x14:id>
+          <x14:id>{01DF0450-3734-4626-8CC9-09B5184BD865}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{759CDCC4-A548-429E-974A-808A28EFB8FC}</x14:id>
+          <x14:id>{E319875B-BB95-4206-9CD2-A0B74CF24A0C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D5B1C543-A861-44A8-80B4-85670AA1D666}</x14:id>
+          <x14:id>{D5A2A30B-8DFA-411A-BA44-3293EC5026EB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{127C0B17-8994-45FA-8363-20555E55FD77}">
+          <x14:cfRule type="dataBar" id="{0E3ABD57-7597-4A6F-A9CF-B218657A67B4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6AF82B66-A67E-4644-A5D9-09BA219ADA00}">
+          <x14:cfRule type="dataBar" id="{01DF0450-3734-4626-8CC9-09B5184BD865}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{759CDCC4-A548-429E-974A-808A28EFB8FC}">
+          <x14:cfRule type="dataBar" id="{E319875B-BB95-4206-9CD2-A0B74CF24A0C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D5B1C543-A861-44A8-80B4-85670AA1D666}">
+          <x14:cfRule type="dataBar" id="{D5A2A30B-8DFA-411A-BA44-3293EC5026EB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{25D9CEDA-CD9F-4E46-8ED0-45C1A4303DCF}</x14:id>
+          <x14:id>{A1648346-6E83-4A8F-9A16-78D950CB2085}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2AFE3761-29A1-4DC7-BC35-BAB65A532456}</x14:id>
+          <x14:id>{9360847B-15A0-4F36-B2AF-AE4D9413D6CF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{484EF240-57E1-4DBE-8676-7E0E49569E5F}</x14:id>
+          <x14:id>{90DE71FE-2322-4660-956D-9B76D57C4B57}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8C483254-A6E4-499A-AB4C-A642BF0493D1}</x14:id>
+          <x14:id>{79C74561-EACF-4C42-BBA5-F0464B935546}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{25D9CEDA-CD9F-4E46-8ED0-45C1A4303DCF}">
+          <x14:cfRule type="dataBar" id="{A1648346-6E83-4A8F-9A16-78D950CB2085}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2AFE3761-29A1-4DC7-BC35-BAB65A532456}">
+          <x14:cfRule type="dataBar" id="{9360847B-15A0-4F36-B2AF-AE4D9413D6CF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{484EF240-57E1-4DBE-8676-7E0E49569E5F}">
+          <x14:cfRule type="dataBar" id="{90DE71FE-2322-4660-956D-9B76D57C4B57}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8C483254-A6E4-499A-AB4C-A642BF0493D1}">
+          <x14:cfRule type="dataBar" id="{79C74561-EACF-4C42-BBA5-F0464B935546}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0E3ABD57-7597-4A6F-A9CF-B218657A67B4}</x14:id>
+          <x14:id>{08CB98FA-E6B4-413C-861C-325EF39CCA84}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{01DF0450-3734-4626-8CC9-09B5184BD865}</x14:id>
+          <x14:id>{26799EB5-D38A-409A-A55E-AFA57293A9FB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E319875B-BB95-4206-9CD2-A0B74CF24A0C}</x14:id>
+          <x14:id>{66B4382B-769D-49CA-A75B-C3342BFBF14D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D5A2A30B-8DFA-411A-BA44-3293EC5026EB}</x14:id>
+          <x14:id>{8D0A863A-17C9-41BA-9103-50468B8E74CA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0E3ABD57-7597-4A6F-A9CF-B218657A67B4}">
+          <x14:cfRule type="dataBar" id="{08CB98FA-E6B4-413C-861C-325EF39CCA84}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{01DF0450-3734-4626-8CC9-09B5184BD865}">
+          <x14:cfRule type="dataBar" id="{26799EB5-D38A-409A-A55E-AFA57293A9FB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E319875B-BB95-4206-9CD2-A0B74CF24A0C}">
+          <x14:cfRule type="dataBar" id="{66B4382B-769D-49CA-A75B-C3342BFBF14D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D5A2A30B-8DFA-411A-BA44-3293EC5026EB}">
+          <x14:cfRule type="dataBar" id="{8D0A863A-17C9-41BA-9103-50468B8E74CA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A1648346-6E83-4A8F-9A16-78D950CB2085}</x14:id>
+          <x14:id>{436742C2-B79B-4F6F-BDC4-FECC8CF6AE6D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9360847B-15A0-4F36-B2AF-AE4D9413D6CF}</x14:id>
+          <x14:id>{4D221361-32F3-423B-AC62-AED5E4316208}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{90DE71FE-2322-4660-956D-9B76D57C4B57}</x14:id>
+          <x14:id>{5BE6A06C-A16C-422F-90F3-401A576A83F9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{79C74561-EACF-4C42-BBA5-F0464B935546}</x14:id>
+          <x14:id>{1A753885-1BA1-442A-850A-DB22E6D11ED5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A1648346-6E83-4A8F-9A16-78D950CB2085}">
+          <x14:cfRule type="dataBar" id="{436742C2-B79B-4F6F-BDC4-FECC8CF6AE6D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9360847B-15A0-4F36-B2AF-AE4D9413D6CF}">
+          <x14:cfRule type="dataBar" id="{4D221361-32F3-423B-AC62-AED5E4316208}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{90DE71FE-2322-4660-956D-9B76D57C4B57}">
+          <x14:cfRule type="dataBar" id="{5BE6A06C-A16C-422F-90F3-401A576A83F9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{79C74561-EACF-4C42-BBA5-F0464B935546}">
+          <x14:cfRule type="dataBar" id="{1A753885-1BA1-442A-850A-DB22E6D11ED5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{08CB98FA-E6B4-413C-861C-325EF39CCA84}</x14:id>
+          <x14:id>{068ECF6E-3F51-48F2-AB1F-B81F308ED48D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{26799EB5-D38A-409A-A55E-AFA57293A9FB}</x14:id>
+          <x14:id>{C5A10B55-EF08-4025-9E50-4F22C64F0938}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{66B4382B-769D-49CA-A75B-C3342BFBF14D}</x14:id>
+          <x14:id>{C862771F-32F2-4D00-A8F7-3CE5CEF09C30}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8D0A863A-17C9-41BA-9103-50468B8E74CA}</x14:id>
+          <x14:id>{F8E58113-CDF2-4E3B-B9E9-3D0DEEEEB20D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{08CB98FA-E6B4-413C-861C-325EF39CCA84}">
+          <x14:cfRule type="dataBar" id="{068ECF6E-3F51-48F2-AB1F-B81F308ED48D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{26799EB5-D38A-409A-A55E-AFA57293A9FB}">
+          <x14:cfRule type="dataBar" id="{C5A10B55-EF08-4025-9E50-4F22C64F0938}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{66B4382B-769D-49CA-A75B-C3342BFBF14D}">
+          <x14:cfRule type="dataBar" id="{C862771F-32F2-4D00-A8F7-3CE5CEF09C30}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8D0A863A-17C9-41BA-9103-50468B8E74CA}">
+          <x14:cfRule type="dataBar" id="{F8E58113-CDF2-4E3B-B9E9-3D0DEEEEB20D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{436742C2-B79B-4F6F-BDC4-FECC8CF6AE6D}</x14:id>
+          <x14:id>{3F1D4512-1244-4599-B1B2-91AAB4BBA0B8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4D221361-32F3-423B-AC62-AED5E4316208}</x14:id>
+          <x14:id>{EE2BF886-7F0B-490C-BF6A-3268F981E05D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5BE6A06C-A16C-422F-90F3-401A576A83F9}</x14:id>
+          <x14:id>{62EDBAD8-E6C8-466D-B373-381A941FBCD0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1A753885-1BA1-442A-850A-DB22E6D11ED5}</x14:id>
+          <x14:id>{CC9C1133-8456-45C9-92A2-28764DF44DDF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{436742C2-B79B-4F6F-BDC4-FECC8CF6AE6D}">
+          <x14:cfRule type="dataBar" id="{3F1D4512-1244-4599-B1B2-91AAB4BBA0B8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4D221361-32F3-423B-AC62-AED5E4316208}">
+          <x14:cfRule type="dataBar" id="{EE2BF886-7F0B-490C-BF6A-3268F981E05D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5BE6A06C-A16C-422F-90F3-401A576A83F9}">
+          <x14:cfRule type="dataBar" id="{62EDBAD8-E6C8-466D-B373-381A941FBCD0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1A753885-1BA1-442A-850A-DB22E6D11ED5}">
+          <x14:cfRule type="dataBar" id="{CC9C1133-8456-45C9-92A2-28764DF44DDF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{068ECF6E-3F51-48F2-AB1F-B81F308ED48D}</x14:id>
+          <x14:id>{DD0B16E7-A8BE-47F4-9933-5B7DD358ACEF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C5A10B55-EF08-4025-9E50-4F22C64F0938}</x14:id>
+          <x14:id>{3A698301-EE4B-40E7-ACC2-460BB0342E69}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C862771F-32F2-4D00-A8F7-3CE5CEF09C30}</x14:id>
+          <x14:id>{66994567-1E46-40BF-ACEB-717EDBEEB1EC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F8E58113-CDF2-4E3B-B9E9-3D0DEEEEB20D}</x14:id>
+          <x14:id>{74A895CD-1027-41B4-BBA2-780CEC1A2587}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{068ECF6E-3F51-48F2-AB1F-B81F308ED48D}">
+          <x14:cfRule type="dataBar" id="{DD0B16E7-A8BE-47F4-9933-5B7DD358ACEF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C5A10B55-EF08-4025-9E50-4F22C64F0938}">
+          <x14:cfRule type="dataBar" id="{3A698301-EE4B-40E7-ACC2-460BB0342E69}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C862771F-32F2-4D00-A8F7-3CE5CEF09C30}">
+          <x14:cfRule type="dataBar" id="{66994567-1E46-40BF-ACEB-717EDBEEB1EC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F8E58113-CDF2-4E3B-B9E9-3D0DEEEEB20D}">
+          <x14:cfRule type="dataBar" id="{74A895CD-1027-41B4-BBA2-780CEC1A2587}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3F1D4512-1244-4599-B1B2-91AAB4BBA0B8}</x14:id>
+          <x14:id>{77536ED2-1DC7-469A-AB1E-4C28D7C4FD31}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EE2BF886-7F0B-490C-BF6A-3268F981E05D}</x14:id>
+          <x14:id>{58CE24A4-273C-459E-B632-8E7D982483D6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{62EDBAD8-E6C8-466D-B373-381A941FBCD0}</x14:id>
+          <x14:id>{07C68F7B-887E-40DC-9F9E-DA5C5720EE86}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CC9C1133-8456-45C9-92A2-28764DF44DDF}</x14:id>
+          <x14:id>{C74BBF1A-A763-43BD-B23E-FCE79427C692}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3F1D4512-1244-4599-B1B2-91AAB4BBA0B8}">
+          <x14:cfRule type="dataBar" id="{77536ED2-1DC7-469A-AB1E-4C28D7C4FD31}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EE2BF886-7F0B-490C-BF6A-3268F981E05D}">
+          <x14:cfRule type="dataBar" id="{58CE24A4-273C-459E-B632-8E7D982483D6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{62EDBAD8-E6C8-466D-B373-381A941FBCD0}">
+          <x14:cfRule type="dataBar" id="{07C68F7B-887E-40DC-9F9E-DA5C5720EE86}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CC9C1133-8456-45C9-92A2-28764DF44DDF}">
+          <x14:cfRule type="dataBar" id="{C74BBF1A-A763-43BD-B23E-FCE79427C692}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 08:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DD0B16E7-A8BE-47F4-9933-5B7DD358ACEF}</x14:id>
+          <x14:id>{3CA99DD7-F702-4473-A4A8-684B3CEB1BFA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3A698301-EE4B-40E7-ACC2-460BB0342E69}</x14:id>
+          <x14:id>{3CDE72C6-7281-49DD-8626-D89A45C3F890}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{66994567-1E46-40BF-ACEB-717EDBEEB1EC}</x14:id>
+          <x14:id>{9F05C52C-A978-41D7-845F-F446E1F9EE00}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{74A895CD-1027-41B4-BBA2-780CEC1A2587}</x14:id>
+          <x14:id>{58763A29-B060-412D-9FFD-7CFC1E849A19}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DD0B16E7-A8BE-47F4-9933-5B7DD358ACEF}">
+          <x14:cfRule type="dataBar" id="{3CA99DD7-F702-4473-A4A8-684B3CEB1BFA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3A698301-EE4B-40E7-ACC2-460BB0342E69}">
+          <x14:cfRule type="dataBar" id="{3CDE72C6-7281-49DD-8626-D89A45C3F890}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{66994567-1E46-40BF-ACEB-717EDBEEB1EC}">
+          <x14:cfRule type="dataBar" id="{9F05C52C-A978-41D7-845F-F446E1F9EE00}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{74A895CD-1027-41B4-BBA2-780CEC1A2587}">
+          <x14:cfRule type="dataBar" id="{58763A29-B060-412D-9FFD-7CFC1E849A19}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{77536ED2-1DC7-469A-AB1E-4C28D7C4FD31}</x14:id>
+          <x14:id>{683A6A50-01A9-4755-B6F2-E8AB0645FD1B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{58CE24A4-273C-459E-B632-8E7D982483D6}</x14:id>
+          <x14:id>{A2876F03-57FE-4290-BE5B-AEFB57CE1CBD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{07C68F7B-887E-40DC-9F9E-DA5C5720EE86}</x14:id>
+          <x14:id>{C1D8E95A-39B2-4EC7-8E9F-63F9FEA10133}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C74BBF1A-A763-43BD-B23E-FCE79427C692}</x14:id>
+          <x14:id>{4C48DBC2-B8D4-4D6A-B72E-E1497C3CFFEF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{77536ED2-1DC7-469A-AB1E-4C28D7C4FD31}">
+          <x14:cfRule type="dataBar" id="{683A6A50-01A9-4755-B6F2-E8AB0645FD1B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{58CE24A4-273C-459E-B632-8E7D982483D6}">
+          <x14:cfRule type="dataBar" id="{A2876F03-57FE-4290-BE5B-AEFB57CE1CBD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{07C68F7B-887E-40DC-9F9E-DA5C5720EE86}">
+          <x14:cfRule type="dataBar" id="{C1D8E95A-39B2-4EC7-8E9F-63F9FEA10133}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C74BBF1A-A763-43BD-B23E-FCE79427C692}">
+          <x14:cfRule type="dataBar" id="{4C48DBC2-B8D4-4D6A-B72E-E1497C3CFFEF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3CA99DD7-F702-4473-A4A8-684B3CEB1BFA}</x14:id>
+          <x14:id>{C188521F-BEDC-4CE0-AED4-34492F17E42A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3CDE72C6-7281-49DD-8626-D89A45C3F890}</x14:id>
+          <x14:id>{E2E0C249-99DE-4A2D-946F-CF2F535A7F83}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9F05C52C-A978-41D7-845F-F446E1F9EE00}</x14:id>
+          <x14:id>{2D8476FF-DD02-4E23-81F5-1B5E31724AE3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{58763A29-B060-412D-9FFD-7CFC1E849A19}</x14:id>
+          <x14:id>{C50C0235-7EB7-4BFA-9D38-D46019DA2F4F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3CA99DD7-F702-4473-A4A8-684B3CEB1BFA}">
+          <x14:cfRule type="dataBar" id="{C188521F-BEDC-4CE0-AED4-34492F17E42A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3CDE72C6-7281-49DD-8626-D89A45C3F890}">
+          <x14:cfRule type="dataBar" id="{E2E0C249-99DE-4A2D-946F-CF2F535A7F83}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9F05C52C-A978-41D7-845F-F446E1F9EE00}">
+          <x14:cfRule type="dataBar" id="{2D8476FF-DD02-4E23-81F5-1B5E31724AE3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{58763A29-B060-412D-9FFD-7CFC1E849A19}">
+          <x14:cfRule type="dataBar" id="{C50C0235-7EB7-4BFA-9D38-D46019DA2F4F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{683A6A50-01A9-4755-B6F2-E8AB0645FD1B}</x14:id>
+          <x14:id>{8E8CEC12-0AC2-49CA-8FB0-1E8237D58284}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A2876F03-57FE-4290-BE5B-AEFB57CE1CBD}</x14:id>
+          <x14:id>{AE4E33AB-D177-4217-8AB9-00855055536C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C1D8E95A-39B2-4EC7-8E9F-63F9FEA10133}</x14:id>
+          <x14:id>{FF764664-43FE-40EF-880F-D1ED6660CA43}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4C48DBC2-B8D4-4D6A-B72E-E1497C3CFFEF}</x14:id>
+          <x14:id>{84C85788-3112-4959-BCDC-B31AECC5BF45}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{683A6A50-01A9-4755-B6F2-E8AB0645FD1B}">
+          <x14:cfRule type="dataBar" id="{8E8CEC12-0AC2-49CA-8FB0-1E8237D58284}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A2876F03-57FE-4290-BE5B-AEFB57CE1CBD}">
+          <x14:cfRule type="dataBar" id="{AE4E33AB-D177-4217-8AB9-00855055536C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C1D8E95A-39B2-4EC7-8E9F-63F9FEA10133}">
+          <x14:cfRule type="dataBar" id="{FF764664-43FE-40EF-880F-D1ED6660CA43}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4C48DBC2-B8D4-4D6A-B72E-E1497C3CFFEF}">
+          <x14:cfRule type="dataBar" id="{84C85788-3112-4959-BCDC-B31AECC5BF45}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C188521F-BEDC-4CE0-AED4-34492F17E42A}</x14:id>
+          <x14:id>{F18D02A2-F92E-4DE3-B45E-E0F797C9107D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E2E0C249-99DE-4A2D-946F-CF2F535A7F83}</x14:id>
+          <x14:id>{2BA31F5D-1BBB-4570-A883-B2EDEFF8669B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2D8476FF-DD02-4E23-81F5-1B5E31724AE3}</x14:id>
+          <x14:id>{EC439318-32EB-4A10-91ED-212DCD2996EF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C50C0235-7EB7-4BFA-9D38-D46019DA2F4F}</x14:id>
+          <x14:id>{4B647B9C-017C-4D98-980B-EB0548911849}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C188521F-BEDC-4CE0-AED4-34492F17E42A}">
+          <x14:cfRule type="dataBar" id="{F18D02A2-F92E-4DE3-B45E-E0F797C9107D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E2E0C249-99DE-4A2D-946F-CF2F535A7F83}">
+          <x14:cfRule type="dataBar" id="{2BA31F5D-1BBB-4570-A883-B2EDEFF8669B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2D8476FF-DD02-4E23-81F5-1B5E31724AE3}">
+          <x14:cfRule type="dataBar" id="{EC439318-32EB-4A10-91ED-212DCD2996EF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C50C0235-7EB7-4BFA-9D38-D46019DA2F4F}">
+          <x14:cfRule type="dataBar" id="{4B647B9C-017C-4D98-980B-EB0548911849}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8E8CEC12-0AC2-49CA-8FB0-1E8237D58284}</x14:id>
+          <x14:id>{28D5277B-AC37-4E42-9620-0B66A04642DF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AE4E33AB-D177-4217-8AB9-00855055536C}</x14:id>
+          <x14:id>{5378D5B8-2069-42BA-A941-A481F2505BC8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FF764664-43FE-40EF-880F-D1ED6660CA43}</x14:id>
+          <x14:id>{8AE4D4C8-575B-4C66-8A9A-6A32FD7AB35C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{84C85788-3112-4959-BCDC-B31AECC5BF45}</x14:id>
+          <x14:id>{1163B5F8-43BE-4E3D-A772-EF662F1BA75A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8E8CEC12-0AC2-49CA-8FB0-1E8237D58284}">
+          <x14:cfRule type="dataBar" id="{28D5277B-AC37-4E42-9620-0B66A04642DF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AE4E33AB-D177-4217-8AB9-00855055536C}">
+          <x14:cfRule type="dataBar" id="{5378D5B8-2069-42BA-A941-A481F2505BC8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FF764664-43FE-40EF-880F-D1ED6660CA43}">
+          <x14:cfRule type="dataBar" id="{8AE4D4C8-575B-4C66-8A9A-6A32FD7AB35C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{84C85788-3112-4959-BCDC-B31AECC5BF45}">
+          <x14:cfRule type="dataBar" id="{1163B5F8-43BE-4E3D-A772-EF662F1BA75A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F18D02A2-F92E-4DE3-B45E-E0F797C9107D}</x14:id>
+          <x14:id>{ACF3FEC7-B438-4217-9D61-FDFFEDC50E81}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2BA31F5D-1BBB-4570-A883-B2EDEFF8669B}</x14:id>
+          <x14:id>{792C9B81-EBDE-493E-8E66-E9BAC94E9ED1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EC439318-32EB-4A10-91ED-212DCD2996EF}</x14:id>
+          <x14:id>{BEB85651-464D-42E3-AA00-74DBEEA3F7C6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4B647B9C-017C-4D98-980B-EB0548911849}</x14:id>
+          <x14:id>{7EEBC536-0159-4538-9891-DA7179ACD628}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F18D02A2-F92E-4DE3-B45E-E0F797C9107D}">
+          <x14:cfRule type="dataBar" id="{ACF3FEC7-B438-4217-9D61-FDFFEDC50E81}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2BA31F5D-1BBB-4570-A883-B2EDEFF8669B}">
+          <x14:cfRule type="dataBar" id="{792C9B81-EBDE-493E-8E66-E9BAC94E9ED1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EC439318-32EB-4A10-91ED-212DCD2996EF}">
+          <x14:cfRule type="dataBar" id="{BEB85651-464D-42E3-AA00-74DBEEA3F7C6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4B647B9C-017C-4D98-980B-EB0548911849}">
+          <x14:cfRule type="dataBar" id="{7EEBC536-0159-4538-9891-DA7179ACD628}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{28D5277B-AC37-4E42-9620-0B66A04642DF}</x14:id>
+          <x14:id>{856631B3-7645-4375-B9AB-ECEF26BA520F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5378D5B8-2069-42BA-A941-A481F2505BC8}</x14:id>
+          <x14:id>{24153C84-0650-4C54-9E0E-BA415940AEEA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8AE4D4C8-575B-4C66-8A9A-6A32FD7AB35C}</x14:id>
+          <x14:id>{366B6701-C916-4606-947C-F12279C6B8F5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1163B5F8-43BE-4E3D-A772-EF662F1BA75A}</x14:id>
+          <x14:id>{799592F9-614B-4CCC-8805-C2753DF892EC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{28D5277B-AC37-4E42-9620-0B66A04642DF}">
+          <x14:cfRule type="dataBar" id="{856631B3-7645-4375-B9AB-ECEF26BA520F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5378D5B8-2069-42BA-A941-A481F2505BC8}">
+          <x14:cfRule type="dataBar" id="{24153C84-0650-4C54-9E0E-BA415940AEEA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8AE4D4C8-575B-4C66-8A9A-6A32FD7AB35C}">
+          <x14:cfRule type="dataBar" id="{366B6701-C916-4606-947C-F12279C6B8F5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1163B5F8-43BE-4E3D-A772-EF662F1BA75A}">
+          <x14:cfRule type="dataBar" id="{799592F9-614B-4CCC-8805-C2753DF892EC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ACF3FEC7-B438-4217-9D61-FDFFEDC50E81}</x14:id>
+          <x14:id>{65E9EBE6-23FC-4F9F-A61C-4127E9F25922}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{792C9B81-EBDE-493E-8E66-E9BAC94E9ED1}</x14:id>
+          <x14:id>{D7F82E04-6369-480F-9472-C1187B4817ED}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BEB85651-464D-42E3-AA00-74DBEEA3F7C6}</x14:id>
+          <x14:id>{441A6EEF-5B25-4301-8EB5-1524917B5C3E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7EEBC536-0159-4538-9891-DA7179ACD628}</x14:id>
+          <x14:id>{B965ED85-273D-468E-958C-C0A066576C81}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ACF3FEC7-B438-4217-9D61-FDFFEDC50E81}">
+          <x14:cfRule type="dataBar" id="{65E9EBE6-23FC-4F9F-A61C-4127E9F25922}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{792C9B81-EBDE-493E-8E66-E9BAC94E9ED1}">
+          <x14:cfRule type="dataBar" id="{D7F82E04-6369-480F-9472-C1187B4817ED}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BEB85651-464D-42E3-AA00-74DBEEA3F7C6}">
+          <x14:cfRule type="dataBar" id="{441A6EEF-5B25-4301-8EB5-1524917B5C3E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7EEBC536-0159-4538-9891-DA7179ACD628}">
+          <x14:cfRule type="dataBar" id="{B965ED85-273D-468E-958C-C0A066576C81}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{856631B3-7645-4375-B9AB-ECEF26BA520F}</x14:id>
+          <x14:id>{C0E5734E-9427-46C2-BC49-63940515E419}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{24153C84-0650-4C54-9E0E-BA415940AEEA}</x14:id>
+          <x14:id>{B964A17A-A0AB-4623-985C-3345DA85CF25}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{366B6701-C916-4606-947C-F12279C6B8F5}</x14:id>
+          <x14:id>{ADAD01BF-76B7-4305-AF5B-DEED3C399D22}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{799592F9-614B-4CCC-8805-C2753DF892EC}</x14:id>
+          <x14:id>{55A56203-9051-4FAF-97A4-A66B138F6296}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{856631B3-7645-4375-B9AB-ECEF26BA520F}">
+          <x14:cfRule type="dataBar" id="{C0E5734E-9427-46C2-BC49-63940515E419}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{24153C84-0650-4C54-9E0E-BA415940AEEA}">
+          <x14:cfRule type="dataBar" id="{B964A17A-A0AB-4623-985C-3345DA85CF25}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{366B6701-C916-4606-947C-F12279C6B8F5}">
+          <x14:cfRule type="dataBar" id="{ADAD01BF-76B7-4305-AF5B-DEED3C399D22}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{799592F9-614B-4CCC-8805-C2753DF892EC}">
+          <x14:cfRule type="dataBar" id="{55A56203-9051-4FAF-97A4-A66B138F6296}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{65E9EBE6-23FC-4F9F-A61C-4127E9F25922}</x14:id>
+          <x14:id>{C94FDFF7-5878-408F-ADF5-39627384BE4B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D7F82E04-6369-480F-9472-C1187B4817ED}</x14:id>
+          <x14:id>{0184FCC3-712D-4D05-BDB8-26F2BF286249}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{441A6EEF-5B25-4301-8EB5-1524917B5C3E}</x14:id>
+          <x14:id>{C4A4BDAF-A540-48FE-98F8-479A282A247E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B965ED85-273D-468E-958C-C0A066576C81}</x14:id>
+          <x14:id>{D5ADFA96-5746-4FBA-8BAB-4C390E44A029}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{65E9EBE6-23FC-4F9F-A61C-4127E9F25922}">
+          <x14:cfRule type="dataBar" id="{C94FDFF7-5878-408F-ADF5-39627384BE4B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D7F82E04-6369-480F-9472-C1187B4817ED}">
+          <x14:cfRule type="dataBar" id="{0184FCC3-712D-4D05-BDB8-26F2BF286249}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{441A6EEF-5B25-4301-8EB5-1524917B5C3E}">
+          <x14:cfRule type="dataBar" id="{C4A4BDAF-A540-48FE-98F8-479A282A247E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B965ED85-273D-468E-958C-C0A066576C81}">
+          <x14:cfRule type="dataBar" id="{D5ADFA96-5746-4FBA-8BAB-4C390E44A029}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C0E5734E-9427-46C2-BC49-63940515E419}</x14:id>
+          <x14:id>{7F811E47-4968-4F4D-92F0-C8D7454EAD7C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B964A17A-A0AB-4623-985C-3345DA85CF25}</x14:id>
+          <x14:id>{17F9A738-6ADF-4664-A04C-0DB101CC75E6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ADAD01BF-76B7-4305-AF5B-DEED3C399D22}</x14:id>
+          <x14:id>{9EB14930-70C4-4B4D-BEED-5168C9E41525}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{55A56203-9051-4FAF-97A4-A66B138F6296}</x14:id>
+          <x14:id>{696C3A41-77D1-4CD3-B5B2-8AA7E3FE42AF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C0E5734E-9427-46C2-BC49-63940515E419}">
+          <x14:cfRule type="dataBar" id="{7F811E47-4968-4F4D-92F0-C8D7454EAD7C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B964A17A-A0AB-4623-985C-3345DA85CF25}">
+          <x14:cfRule type="dataBar" id="{17F9A738-6ADF-4664-A04C-0DB101CC75E6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ADAD01BF-76B7-4305-AF5B-DEED3C399D22}">
+          <x14:cfRule type="dataBar" id="{9EB14930-70C4-4B4D-BEED-5168C9E41525}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{55A56203-9051-4FAF-97A4-A66B138F6296}">
+          <x14:cfRule type="dataBar" id="{696C3A41-77D1-4CD3-B5B2-8AA7E3FE42AF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C94FDFF7-5878-408F-ADF5-39627384BE4B}</x14:id>
+          <x14:id>{DFC8DECD-1BBD-4762-A09F-88BD2802E950}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0184FCC3-712D-4D05-BDB8-26F2BF286249}</x14:id>
+          <x14:id>{3E4D066C-22E3-457E-A6BD-1AD5CF065D3E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C4A4BDAF-A540-48FE-98F8-479A282A247E}</x14:id>
+          <x14:id>{A81AAAD3-6C4F-4DBE-96D0-1FAD95DA2B5C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D5ADFA96-5746-4FBA-8BAB-4C390E44A029}</x14:id>
+          <x14:id>{1535306A-85FF-4633-8CA3-A619EE699FEA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C94FDFF7-5878-408F-ADF5-39627384BE4B}">
+          <x14:cfRule type="dataBar" id="{DFC8DECD-1BBD-4762-A09F-88BD2802E950}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0184FCC3-712D-4D05-BDB8-26F2BF286249}">
+          <x14:cfRule type="dataBar" id="{3E4D066C-22E3-457E-A6BD-1AD5CF065D3E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C4A4BDAF-A540-48FE-98F8-479A282A247E}">
+          <x14:cfRule type="dataBar" id="{A81AAAD3-6C4F-4DBE-96D0-1FAD95DA2B5C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D5ADFA96-5746-4FBA-8BAB-4C390E44A029}">
+          <x14:cfRule type="dataBar" id="{1535306A-85FF-4633-8CA3-A619EE699FEA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F811E47-4968-4F4D-92F0-C8D7454EAD7C}</x14:id>
+          <x14:id>{4448CD7C-1543-43E4-8CDD-A659E9E306D6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{17F9A738-6ADF-4664-A04C-0DB101CC75E6}</x14:id>
+          <x14:id>{A394F650-EF04-412C-92DC-0B42659CE427}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9EB14930-70C4-4B4D-BEED-5168C9E41525}</x14:id>
+          <x14:id>{9164A4A5-1C3A-49DF-BFD3-7A0AEEDE05C3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{696C3A41-77D1-4CD3-B5B2-8AA7E3FE42AF}</x14:id>
+          <x14:id>{369ACC7A-784F-4ABC-8DDD-DB5D4D67ADC4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F811E47-4968-4F4D-92F0-C8D7454EAD7C}">
+          <x14:cfRule type="dataBar" id="{4448CD7C-1543-43E4-8CDD-A659E9E306D6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{17F9A738-6ADF-4664-A04C-0DB101CC75E6}">
+          <x14:cfRule type="dataBar" id="{A394F650-EF04-412C-92DC-0B42659CE427}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9EB14930-70C4-4B4D-BEED-5168C9E41525}">
+          <x14:cfRule type="dataBar" id="{9164A4A5-1C3A-49DF-BFD3-7A0AEEDE05C3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{696C3A41-77D1-4CD3-B5B2-8AA7E3FE42AF}">
+          <x14:cfRule type="dataBar" id="{369ACC7A-784F-4ABC-8DDD-DB5D4D67ADC4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DFC8DECD-1BBD-4762-A09F-88BD2802E950}</x14:id>
+          <x14:id>{53CFA013-82C3-4CF7-AFFC-48D03A9E4FAC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3E4D066C-22E3-457E-A6BD-1AD5CF065D3E}</x14:id>
+          <x14:id>{62B179B4-3433-44DF-9F7F-37EC25AA80D1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A81AAAD3-6C4F-4DBE-96D0-1FAD95DA2B5C}</x14:id>
+          <x14:id>{FD25607A-2E71-416B-95B7-C48B86BF9A35}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1535306A-85FF-4633-8CA3-A619EE699FEA}</x14:id>
+          <x14:id>{4574D1F3-24C7-42EB-8F6B-E8E0CEF3B3FE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DFC8DECD-1BBD-4762-A09F-88BD2802E950}">
+          <x14:cfRule type="dataBar" id="{53CFA013-82C3-4CF7-AFFC-48D03A9E4FAC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3E4D066C-22E3-457E-A6BD-1AD5CF065D3E}">
+          <x14:cfRule type="dataBar" id="{62B179B4-3433-44DF-9F7F-37EC25AA80D1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A81AAAD3-6C4F-4DBE-96D0-1FAD95DA2B5C}">
+          <x14:cfRule type="dataBar" id="{FD25607A-2E71-416B-95B7-C48B86BF9A35}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1535306A-85FF-4633-8CA3-A619EE699FEA}">
+          <x14:cfRule type="dataBar" id="{4574D1F3-24C7-42EB-8F6B-E8E0CEF3B3FE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4448CD7C-1543-43E4-8CDD-A659E9E306D6}</x14:id>
+          <x14:id>{BAA7E27D-1ABE-4E6A-9879-45E018DF3049}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A394F650-EF04-412C-92DC-0B42659CE427}</x14:id>
+          <x14:id>{7F749574-6B24-466B-8CDE-1A2186AC3AE9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9164A4A5-1C3A-49DF-BFD3-7A0AEEDE05C3}</x14:id>
+          <x14:id>{2E24C637-9EA1-47A8-86B8-C3EC98C9AAF0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{369ACC7A-784F-4ABC-8DDD-DB5D4D67ADC4}</x14:id>
+          <x14:id>{88612E03-BB6A-4338-BA7F-1AAFDDDABD48}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4448CD7C-1543-43E4-8CDD-A659E9E306D6}">
+          <x14:cfRule type="dataBar" id="{BAA7E27D-1ABE-4E6A-9879-45E018DF3049}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A394F650-EF04-412C-92DC-0B42659CE427}">
+          <x14:cfRule type="dataBar" id="{7F749574-6B24-466B-8CDE-1A2186AC3AE9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9164A4A5-1C3A-49DF-BFD3-7A0AEEDE05C3}">
+          <x14:cfRule type="dataBar" id="{2E24C637-9EA1-47A8-86B8-C3EC98C9AAF0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{369ACC7A-784F-4ABC-8DDD-DB5D4D67ADC4}">
+          <x14:cfRule type="dataBar" id="{88612E03-BB6A-4338-BA7F-1AAFDDDABD48}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{53CFA013-82C3-4CF7-AFFC-48D03A9E4FAC}</x14:id>
+          <x14:id>{13BBA3A2-8F26-44C8-BCDB-994C9D3E1F5C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{62B179B4-3433-44DF-9F7F-37EC25AA80D1}</x14:id>
+          <x14:id>{1DC1BE81-F605-44EB-BF2F-FE710939A62F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FD25607A-2E71-416B-95B7-C48B86BF9A35}</x14:id>
+          <x14:id>{782A32E6-195C-404A-B097-1D7D5241F4AF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4574D1F3-24C7-42EB-8F6B-E8E0CEF3B3FE}</x14:id>
+          <x14:id>{4809F1FB-F325-4379-9A70-862777ED604D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{53CFA013-82C3-4CF7-AFFC-48D03A9E4FAC}">
+          <x14:cfRule type="dataBar" id="{13BBA3A2-8F26-44C8-BCDB-994C9D3E1F5C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{62B179B4-3433-44DF-9F7F-37EC25AA80D1}">
+          <x14:cfRule type="dataBar" id="{1DC1BE81-F605-44EB-BF2F-FE710939A62F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FD25607A-2E71-416B-95B7-C48B86BF9A35}">
+          <x14:cfRule type="dataBar" id="{782A32E6-195C-404A-B097-1D7D5241F4AF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4574D1F3-24C7-42EB-8F6B-E8E0CEF3B3FE}">
+          <x14:cfRule type="dataBar" id="{4809F1FB-F325-4379-9A70-862777ED604D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BAA7E27D-1ABE-4E6A-9879-45E018DF3049}</x14:id>
+          <x14:id>{69CFBD5E-4355-4B0D-8A91-022F1FCC1D5B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F749574-6B24-466B-8CDE-1A2186AC3AE9}</x14:id>
+          <x14:id>{FCC0DD90-DFC0-44E5-A420-88B095F2DF85}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2E24C637-9EA1-47A8-86B8-C3EC98C9AAF0}</x14:id>
+          <x14:id>{C6035AE8-2277-4D15-B1DC-763ED61AF12C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{88612E03-BB6A-4338-BA7F-1AAFDDDABD48}</x14:id>
+          <x14:id>{3618DB15-87A5-434A-BC67-84DCFB8FAFCA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BAA7E27D-1ABE-4E6A-9879-45E018DF3049}">
+          <x14:cfRule type="dataBar" id="{69CFBD5E-4355-4B0D-8A91-022F1FCC1D5B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F749574-6B24-466B-8CDE-1A2186AC3AE9}">
+          <x14:cfRule type="dataBar" id="{FCC0DD90-DFC0-44E5-A420-88B095F2DF85}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2E24C637-9EA1-47A8-86B8-C3EC98C9AAF0}">
+          <x14:cfRule type="dataBar" id="{C6035AE8-2277-4D15-B1DC-763ED61AF12C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{88612E03-BB6A-4338-BA7F-1AAFDDDABD48}">
+          <x14:cfRule type="dataBar" id="{3618DB15-87A5-434A-BC67-84DCFB8FAFCA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{13BBA3A2-8F26-44C8-BCDB-994C9D3E1F5C}</x14:id>
+          <x14:id>{7E34453A-3E66-4481-8CE6-96BECB2D46D7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1DC1BE81-F605-44EB-BF2F-FE710939A62F}</x14:id>
+          <x14:id>{7BDB50DD-D80F-4F5B-8570-EDE1E290F50C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{782A32E6-195C-404A-B097-1D7D5241F4AF}</x14:id>
+          <x14:id>{36826C26-68A1-4D14-9077-E6A6DA959CE7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4809F1FB-F325-4379-9A70-862777ED604D}</x14:id>
+          <x14:id>{99E24938-CBB2-45DE-A3A7-312F99366907}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{13BBA3A2-8F26-44C8-BCDB-994C9D3E1F5C}">
+          <x14:cfRule type="dataBar" id="{7E34453A-3E66-4481-8CE6-96BECB2D46D7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1DC1BE81-F605-44EB-BF2F-FE710939A62F}">
+          <x14:cfRule type="dataBar" id="{7BDB50DD-D80F-4F5B-8570-EDE1E290F50C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{782A32E6-195C-404A-B097-1D7D5241F4AF}">
+          <x14:cfRule type="dataBar" id="{36826C26-68A1-4D14-9077-E6A6DA959CE7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4809F1FB-F325-4379-9A70-862777ED604D}">
+          <x14:cfRule type="dataBar" id="{99E24938-CBB2-45DE-A3A7-312F99366907}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{69CFBD5E-4355-4B0D-8A91-022F1FCC1D5B}</x14:id>
+          <x14:id>{82102C04-23D7-4419-AD7A-8733568EA155}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FCC0DD90-DFC0-44E5-A420-88B095F2DF85}</x14:id>
+          <x14:id>{097973B6-E9ED-4A73-9D18-8C0986CFDE79}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C6035AE8-2277-4D15-B1DC-763ED61AF12C}</x14:id>
+          <x14:id>{692A7F5C-91C8-49FC-9AAE-65AE27CDB69E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3618DB15-87A5-434A-BC67-84DCFB8FAFCA}</x14:id>
+          <x14:id>{461AF121-C682-4E13-AD2E-F8AC2B798CF8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{69CFBD5E-4355-4B0D-8A91-022F1FCC1D5B}">
+          <x14:cfRule type="dataBar" id="{82102C04-23D7-4419-AD7A-8733568EA155}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FCC0DD90-DFC0-44E5-A420-88B095F2DF85}">
+          <x14:cfRule type="dataBar" id="{097973B6-E9ED-4A73-9D18-8C0986CFDE79}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C6035AE8-2277-4D15-B1DC-763ED61AF12C}">
+          <x14:cfRule type="dataBar" id="{692A7F5C-91C8-49FC-9AAE-65AE27CDB69E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3618DB15-87A5-434A-BC67-84DCFB8FAFCA}">
+          <x14:cfRule type="dataBar" id="{461AF121-C682-4E13-AD2E-F8AC2B798CF8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7E34453A-3E66-4481-8CE6-96BECB2D46D7}</x14:id>
+          <x14:id>{50F0144D-8163-4420-A2E8-473D5DF6639B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7BDB50DD-D80F-4F5B-8570-EDE1E290F50C}</x14:id>
+          <x14:id>{FD9E27E9-7C33-43EA-AB78-B603DFCC3392}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{36826C26-68A1-4D14-9077-E6A6DA959CE7}</x14:id>
+          <x14:id>{77F1B8A8-266B-466A-A9C9-B7B3911EFB79}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{99E24938-CBB2-45DE-A3A7-312F99366907}</x14:id>
+          <x14:id>{91402D65-6B14-4DD2-9EA6-BEFA4C5C8A88}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7E34453A-3E66-4481-8CE6-96BECB2D46D7}">
+          <x14:cfRule type="dataBar" id="{50F0144D-8163-4420-A2E8-473D5DF6639B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7BDB50DD-D80F-4F5B-8570-EDE1E290F50C}">
+          <x14:cfRule type="dataBar" id="{FD9E27E9-7C33-43EA-AB78-B603DFCC3392}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{36826C26-68A1-4D14-9077-E6A6DA959CE7}">
+          <x14:cfRule type="dataBar" id="{77F1B8A8-266B-466A-A9C9-B7B3911EFB79}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{99E24938-CBB2-45DE-A3A7-312F99366907}">
+          <x14:cfRule type="dataBar" id="{91402D65-6B14-4DD2-9EA6-BEFA4C5C8A88}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{82102C04-23D7-4419-AD7A-8733568EA155}</x14:id>
+          <x14:id>{EC06914E-E061-431E-B0EF-743D8F95F208}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{097973B6-E9ED-4A73-9D18-8C0986CFDE79}</x14:id>
+          <x14:id>{2589F4A4-5ADA-44CD-8110-BADBBE1219CB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{692A7F5C-91C8-49FC-9AAE-65AE27CDB69E}</x14:id>
+          <x14:id>{13CFA858-0088-4CE7-8BFA-B419C70A0E38}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{461AF121-C682-4E13-AD2E-F8AC2B798CF8}</x14:id>
+          <x14:id>{302F1234-F759-4C09-B918-03E545B4545C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{82102C04-23D7-4419-AD7A-8733568EA155}">
+          <x14:cfRule type="dataBar" id="{EC06914E-E061-431E-B0EF-743D8F95F208}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{097973B6-E9ED-4A73-9D18-8C0986CFDE79}">
+          <x14:cfRule type="dataBar" id="{2589F4A4-5ADA-44CD-8110-BADBBE1219CB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{692A7F5C-91C8-49FC-9AAE-65AE27CDB69E}">
+          <x14:cfRule type="dataBar" id="{13CFA858-0088-4CE7-8BFA-B419C70A0E38}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{461AF121-C682-4E13-AD2E-F8AC2B798CF8}">
+          <x14:cfRule type="dataBar" id="{302F1234-F759-4C09-B918-03E545B4545C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{50F0144D-8163-4420-A2E8-473D5DF6639B}</x14:id>
+          <x14:id>{49528EF2-CB50-44B0-A432-7095BCD1EF4B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FD9E27E9-7C33-43EA-AB78-B603DFCC3392}</x14:id>
+          <x14:id>{DE7E20A0-4C8E-41C0-BA49-89A45AEE5F18}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{77F1B8A8-266B-466A-A9C9-B7B3911EFB79}</x14:id>
+          <x14:id>{CCF55341-5352-4FC9-9778-77B3252A75A9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{91402D65-6B14-4DD2-9EA6-BEFA4C5C8A88}</x14:id>
+          <x14:id>{E3C603AB-B070-458A-BB04-EE43F957EC73}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{50F0144D-8163-4420-A2E8-473D5DF6639B}">
+          <x14:cfRule type="dataBar" id="{49528EF2-CB50-44B0-A432-7095BCD1EF4B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FD9E27E9-7C33-43EA-AB78-B603DFCC3392}">
+          <x14:cfRule type="dataBar" id="{DE7E20A0-4C8E-41C0-BA49-89A45AEE5F18}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{77F1B8A8-266B-466A-A9C9-B7B3911EFB79}">
+          <x14:cfRule type="dataBar" id="{CCF55341-5352-4FC9-9778-77B3252A75A9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{91402D65-6B14-4DD2-9EA6-BEFA4C5C8A88}">
+          <x14:cfRule type="dataBar" id="{E3C603AB-B070-458A-BB04-EE43F957EC73}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EC06914E-E061-431E-B0EF-743D8F95F208}</x14:id>
+          <x14:id>{40E0F037-CA36-4F9C-9A9C-49FFB7472AA5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2589F4A4-5ADA-44CD-8110-BADBBE1219CB}</x14:id>
+          <x14:id>{1F4F757C-6E1D-4952-834B-665D7E1634C0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{13CFA858-0088-4CE7-8BFA-B419C70A0E38}</x14:id>
+          <x14:id>{2A00C2CF-4892-4D69-A034-71E8F88DA798}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{302F1234-F759-4C09-B918-03E545B4545C}</x14:id>
+          <x14:id>{919A1151-D814-480C-A95B-5608BF05EE39}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EC06914E-E061-431E-B0EF-743D8F95F208}">
+          <x14:cfRule type="dataBar" id="{40E0F037-CA36-4F9C-9A9C-49FFB7472AA5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2589F4A4-5ADA-44CD-8110-BADBBE1219CB}">
+          <x14:cfRule type="dataBar" id="{1F4F757C-6E1D-4952-834B-665D7E1634C0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{13CFA858-0088-4CE7-8BFA-B419C70A0E38}">
+          <x14:cfRule type="dataBar" id="{2A00C2CF-4892-4D69-A034-71E8F88DA798}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{302F1234-F759-4C09-B918-03E545B4545C}">
+          <x14:cfRule type="dataBar" id="{919A1151-D814-480C-A95B-5608BF05EE39}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-16 09:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49528EF2-CB50-44B0-A432-7095BCD1EF4B}</x14:id>
+          <x14:id>{AA7DB267-F9C0-4477-A3F0-793BC42AAC8C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DE7E20A0-4C8E-41C0-BA49-89A45AEE5F18}</x14:id>
+          <x14:id>{31D6C626-0603-49C3-914D-450915F16BA8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CCF55341-5352-4FC9-9778-77B3252A75A9}</x14:id>
+          <x14:id>{ACAB62E7-047F-4531-8C64-8C3FF9A8BBE3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E3C603AB-B070-458A-BB04-EE43F957EC73}</x14:id>
+          <x14:id>{709F9A3D-E866-4670-8452-2F7AFB686FD2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49528EF2-CB50-44B0-A432-7095BCD1EF4B}">
+          <x14:cfRule type="dataBar" id="{AA7DB267-F9C0-4477-A3F0-793BC42AAC8C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DE7E20A0-4C8E-41C0-BA49-89A45AEE5F18}">
+          <x14:cfRule type="dataBar" id="{31D6C626-0603-49C3-914D-450915F16BA8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CCF55341-5352-4FC9-9778-77B3252A75A9}">
+          <x14:cfRule type="dataBar" id="{ACAB62E7-047F-4531-8C64-8C3FF9A8BBE3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E3C603AB-B070-458A-BB04-EE43F957EC73}">
+          <x14:cfRule type="dataBar" id="{709F9A3D-E866-4670-8452-2F7AFB686FD2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{40E0F037-CA36-4F9C-9A9C-49FFB7472AA5}</x14:id>
+          <x14:id>{C649C16D-3A02-4920-996D-57BE5D619492}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1F4F757C-6E1D-4952-834B-665D7E1634C0}</x14:id>
+          <x14:id>{83318872-0FA1-4199-B3B0-F5713C499A43}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2A00C2CF-4892-4D69-A034-71E8F88DA798}</x14:id>
+          <x14:id>{9BB5C69D-5ABB-4DF1-99CF-4119FB16B169}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{919A1151-D814-480C-A95B-5608BF05EE39}</x14:id>
+          <x14:id>{5B8A78FB-AF6F-44D3-9BAF-134D407D05FA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{40E0F037-CA36-4F9C-9A9C-49FFB7472AA5}">
+          <x14:cfRule type="dataBar" id="{C649C16D-3A02-4920-996D-57BE5D619492}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1F4F757C-6E1D-4952-834B-665D7E1634C0}">
+          <x14:cfRule type="dataBar" id="{83318872-0FA1-4199-B3B0-F5713C499A43}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2A00C2CF-4892-4D69-A034-71E8F88DA798}">
+          <x14:cfRule type="dataBar" id="{9BB5C69D-5ABB-4DF1-99CF-4119FB16B169}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{919A1151-D814-480C-A95B-5608BF05EE39}">
+          <x14:cfRule type="dataBar" id="{5B8A78FB-AF6F-44D3-9BAF-134D407D05FA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing 2026-10-16 23:01Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-12.xlsx
+++ b/public/reports/weekly_briefing/2026-10-12.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="46545" yWindow="5250" windowWidth="28800" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="주간 브리핑" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="신고가 근접" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="투자자별 순매수" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="공매도·대차" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="섹터x수급" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="업종별 수급 모멘텀" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="주간 브리핑" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="신고가 근접" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="투자자별 순매수" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공매도·대차" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="섹터x수급" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="업종별 수급 모멘텀" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'신고가 근접'!$A$5:$L$30</definedName>
@@ -1057,7 +1057,7 @@
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>미국 종가 기준 10/09 → 10/15, %</t>
+          <t>미국 종가 기준 10/09 → 10/16, %</t>
         </is>
       </c>
       <c r="I6" s="18" t="inlineStr"/>
@@ -1127,19 +1127,19 @@
         <v>33805</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>-0.86</v>
+        <v>-1.95</v>
       </c>
       <c r="F8" s="28" t="n">
-        <v>1.01</v>
+        <v>0.67</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>-2.39</v>
+        <v>-4.48</v>
       </c>
       <c r="H8" s="28" t="n">
-        <v>10.92</v>
+        <v>34.7</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>-7.88</v>
+        <v>-11.41</v>
       </c>
     </row>
     <row r="9">
@@ -1194,11 +1194,11 @@
       </c>
       <c r="C12" s="31" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>에너지</t>
         </is>
       </c>
       <c r="D12" s="32" t="n">
-        <v>3.74</v>
+        <v>4.86</v>
       </c>
     </row>
     <row r="13">
@@ -1214,11 +1214,11 @@
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t>소재</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="D13" s="32" t="n">
-        <v>2.29</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="14">
@@ -1234,11 +1234,11 @@
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
-          <t>에너지</t>
+          <t>소재</t>
         </is>
       </c>
       <c r="D14" s="32" t="n">
-        <v>2.27</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="15">
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>-7.37</v>
+        <v>-10.53</v>
       </c>
     </row>
     <row r="16">
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="D16" s="33" t="n">
-        <v>-4.82</v>
+        <v>-7.7</v>
       </c>
     </row>
     <row r="17">
@@ -1298,7 +1298,7 @@
         </is>
       </c>
       <c r="D17" s="33" t="n">
-        <v>-2.59</v>
+        <v>-6.15</v>
       </c>
     </row>
     <row r="18">
@@ -12273,7 +12273,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AA7DB267-F9C0-4477-A3F0-793BC42AAC8C}</x14:id>
+          <x14:id>{F8F3B503-BB28-41BE-BD4E-67DA548DE544}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12287,7 +12287,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{31D6C626-0603-49C3-914D-450915F16BA8}</x14:id>
+          <x14:id>{1ECC8459-02A1-4A96-BAA0-DBB7411CF1B0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12301,7 +12301,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ACAB62E7-047F-4531-8C64-8C3FF9A8BBE3}</x14:id>
+          <x14:id>{6220E516-7685-4AAF-90AE-C14354E9BB7F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12315,7 +12315,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{709F9A3D-E866-4670-8452-2F7AFB686FD2}</x14:id>
+          <x14:id>{5142AA4D-FF37-48D5-A87D-92B6E52317BB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12325,7 +12325,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AA7DB267-F9C0-4477-A3F0-793BC42AAC8C}">
+          <x14:cfRule type="dataBar" id="{F8F3B503-BB28-41BE-BD4E-67DA548DE544}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12338,7 +12338,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{31D6C626-0603-49C3-914D-450915F16BA8}">
+          <x14:cfRule type="dataBar" id="{1ECC8459-02A1-4A96-BAA0-DBB7411CF1B0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12351,7 +12351,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ACAB62E7-047F-4531-8C64-8C3FF9A8BBE3}">
+          <x14:cfRule type="dataBar" id="{6220E516-7685-4AAF-90AE-C14354E9BB7F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12364,7 +12364,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{709F9A3D-E866-4670-8452-2F7AFB686FD2}">
+          <x14:cfRule type="dataBar" id="{5142AA4D-FF37-48D5-A87D-92B6E52317BB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27878,7 +27878,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C649C16D-3A02-4920-996D-57BE5D619492}</x14:id>
+          <x14:id>{9C520A6C-0923-4DD6-9783-C2DC3F119F76}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27892,7 +27892,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{83318872-0FA1-4199-B3B0-F5713C499A43}</x14:id>
+          <x14:id>{F63FA0B5-699C-453F-B645-003D14FE3D88}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27906,7 +27906,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9BB5C69D-5ABB-4DF1-99CF-4119FB16B169}</x14:id>
+          <x14:id>{66A0785E-8DA0-4400-BB56-5D9C9E495962}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27920,7 +27920,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5B8A78FB-AF6F-44D3-9BAF-134D407D05FA}</x14:id>
+          <x14:id>{7B086EC0-1E84-46FD-83A5-84065DBB86C2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27930,7 +27930,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C649C16D-3A02-4920-996D-57BE5D619492}">
+          <x14:cfRule type="dataBar" id="{9C520A6C-0923-4DD6-9783-C2DC3F119F76}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27943,7 +27943,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{83318872-0FA1-4199-B3B0-F5713C499A43}">
+          <x14:cfRule type="dataBar" id="{F63FA0B5-699C-453F-B645-003D14FE3D88}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27956,7 +27956,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9BB5C69D-5ABB-4DF1-99CF-4119FB16B169}">
+          <x14:cfRule type="dataBar" id="{66A0785E-8DA0-4400-BB56-5D9C9E495962}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27969,7 +27969,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5B8A78FB-AF6F-44D3-9BAF-134D407D05FA}">
+          <x14:cfRule type="dataBar" id="{7B086EC0-1E84-46FD-83A5-84065DBB86C2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>